<commit_message>
docs: Re-generate Excel control maps to precisely match XML paths and UUIDs
</commit_message>
<xml_diff>
--- a/docs/APC40MKII_Electric_Zentropa_True_Button_Toggles_Map.xlsx
+++ b/docs/APC40MKII_Electric_Zentropa_True_Button_Toggles_Map.xlsx
@@ -13856,11 +13856,7 @@
       <c r="A5" s="71" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="72" t="inlineStr">
-        <is>
-          <t>1784313900056</t>
-        </is>
-      </c>
+      <c r="B5" s="72" t="n"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -13951,11 +13947,7 @@
       <c r="A6" s="71" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="72" t="inlineStr">
-        <is>
-          <t>1784313900001</t>
-        </is>
-      </c>
+      <c r="B6" s="72" t="n"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -14046,11 +14038,7 @@
       <c r="A7" s="71" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="72" t="inlineStr">
-        <is>
-          <t>1784313900042</t>
-        </is>
-      </c>
+      <c r="B7" s="72" t="n"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -14141,11 +14129,7 @@
       <c r="A8" s="71" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="72" t="inlineStr">
-        <is>
-          <t>1784313900041</t>
-        </is>
-      </c>
+      <c r="B8" s="72" t="n"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -14236,11 +14220,7 @@
       <c r="A9" s="71" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="72" t="inlineStr">
-        <is>
-          <t>1784313900007</t>
-        </is>
-      </c>
+      <c r="B9" s="72" t="n"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -14331,11 +14311,7 @@
       <c r="A10" s="71" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="72" t="inlineStr">
-        <is>
-          <t>1784313900005</t>
-        </is>
-      </c>
+      <c r="B10" s="72" t="n"/>
       <c r="C10" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -14426,11 +14402,7 @@
       <c r="A11" s="71" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="72" t="inlineStr">
-        <is>
-          <t>1784313900046</t>
-        </is>
-      </c>
+      <c r="B11" s="72" t="n"/>
       <c r="C11" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -14521,11 +14493,7 @@
       <c r="A12" s="71" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="72" t="inlineStr">
-        <is>
-          <t>1784313900023</t>
-        </is>
-      </c>
+      <c r="B12" s="72" t="n"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -14616,11 +14584,7 @@
       <c r="A13" s="71" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="72" t="inlineStr">
-        <is>
-          <t>1784313900050</t>
-        </is>
-      </c>
+      <c r="B13" s="72" t="n"/>
       <c r="C13" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -14711,11 +14675,7 @@
       <c r="A14" s="71" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="72" t="inlineStr">
-        <is>
-          <t>1784313900024</t>
-        </is>
-      </c>
+      <c r="B14" s="72" t="n"/>
       <c r="C14" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -14806,11 +14766,7 @@
       <c r="A15" s="71" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="72" t="inlineStr">
-        <is>
-          <t>1784313900044</t>
-        </is>
-      </c>
+      <c r="B15" s="72" t="n"/>
       <c r="C15" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -14901,11 +14857,7 @@
       <c r="A16" s="71" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="72" t="inlineStr">
-        <is>
-          <t>1784313900013</t>
-        </is>
-      </c>
+      <c r="B16" s="72" t="n"/>
       <c r="C16" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -14996,11 +14948,7 @@
       <c r="A17" s="71" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="72" t="inlineStr">
-        <is>
-          <t>1784313900045</t>
-        </is>
-      </c>
+      <c r="B17" s="72" t="n"/>
       <c r="C17" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -15091,11 +15039,7 @@
       <c r="A18" s="71" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="72" t="inlineStr">
-        <is>
-          <t>1784313900061</t>
-        </is>
-      </c>
+      <c r="B18" s="72" t="n"/>
       <c r="C18" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -15186,11 +15130,7 @@
       <c r="A19" s="71" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="72" t="inlineStr">
-        <is>
-          <t>1784313900040</t>
-        </is>
-      </c>
+      <c r="B19" s="72" t="n"/>
       <c r="C19" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -15281,11 +15221,7 @@
       <c r="A20" s="71" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="72" t="inlineStr">
-        <is>
-          <t>1784313900012</t>
-        </is>
-      </c>
+      <c r="B20" s="72" t="n"/>
       <c r="C20" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -15376,11 +15312,7 @@
       <c r="A21" s="71" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="72" t="inlineStr">
-        <is>
-          <t>1784313900047</t>
-        </is>
-      </c>
+      <c r="B21" s="72" t="n"/>
       <c r="C21" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -15471,11 +15403,7 @@
       <c r="A22" s="71" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="72" t="inlineStr">
-        <is>
-          <t>1784313900051</t>
-        </is>
-      </c>
+      <c r="B22" s="72" t="n"/>
       <c r="C22" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -15566,11 +15494,7 @@
       <c r="A23" s="71" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="72" t="inlineStr">
-        <is>
-          <t>1784313900055</t>
-        </is>
-      </c>
+      <c r="B23" s="72" t="n"/>
       <c r="C23" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -15661,11 +15585,7 @@
       <c r="A24" s="71" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="72" t="inlineStr">
-        <is>
-          <t>1784313900027</t>
-        </is>
-      </c>
+      <c r="B24" s="72" t="n"/>
       <c r="C24" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -15756,11 +15676,7 @@
       <c r="A25" s="71" t="n">
         <v>21</v>
       </c>
-      <c r="B25" s="72" t="inlineStr">
-        <is>
-          <t>1784313900057</t>
-        </is>
-      </c>
+      <c r="B25" s="72" t="n"/>
       <c r="C25" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -15851,11 +15767,7 @@
       <c r="A26" s="71" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="72" t="inlineStr">
-        <is>
-          <t>1784313900039</t>
-        </is>
-      </c>
+      <c r="B26" s="72" t="n"/>
       <c r="C26" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -15946,11 +15858,7 @@
       <c r="A27" s="71" t="n">
         <v>23</v>
       </c>
-      <c r="B27" s="72" t="inlineStr">
-        <is>
-          <t>1784313900049</t>
-        </is>
-      </c>
+      <c r="B27" s="72" t="n"/>
       <c r="C27" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -16041,11 +15949,7 @@
       <c r="A28" s="71" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="72" t="inlineStr">
-        <is>
-          <t>1784313900037</t>
-        </is>
-      </c>
+      <c r="B28" s="72" t="n"/>
       <c r="C28" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -16136,11 +16040,7 @@
       <c r="A29" s="71" t="n">
         <v>25</v>
       </c>
-      <c r="B29" s="72" t="inlineStr">
-        <is>
-          <t>1784313900022</t>
-        </is>
-      </c>
+      <c r="B29" s="72" t="n"/>
       <c r="C29" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -16231,11 +16131,7 @@
       <c r="A30" s="71" t="n">
         <v>26</v>
       </c>
-      <c r="B30" s="72" t="inlineStr">
-        <is>
-          <t>1784313900032</t>
-        </is>
-      </c>
+      <c r="B30" s="72" t="n"/>
       <c r="C30" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -16326,11 +16222,7 @@
       <c r="A31" s="71" t="n">
         <v>27</v>
       </c>
-      <c r="B31" s="72" t="inlineStr">
-        <is>
-          <t>1784313900031</t>
-        </is>
-      </c>
+      <c r="B31" s="72" t="n"/>
       <c r="C31" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -16421,11 +16313,7 @@
       <c r="A32" s="71" t="n">
         <v>28</v>
       </c>
-      <c r="B32" s="72" t="inlineStr">
-        <is>
-          <t>1784313900019</t>
-        </is>
-      </c>
+      <c r="B32" s="72" t="n"/>
       <c r="C32" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -16516,11 +16404,7 @@
       <c r="A33" s="71" t="n">
         <v>29</v>
       </c>
-      <c r="B33" s="72" t="inlineStr">
-        <is>
-          <t>1784313900054</t>
-        </is>
-      </c>
+      <c r="B33" s="72" t="n"/>
       <c r="C33" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -16611,11 +16495,7 @@
       <c r="A34" s="71" t="n">
         <v>30</v>
       </c>
-      <c r="B34" s="72" t="inlineStr">
-        <is>
-          <t>1784313900017</t>
-        </is>
-      </c>
+      <c r="B34" s="72" t="n"/>
       <c r="C34" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -16706,11 +16586,7 @@
       <c r="A35" s="71" t="n">
         <v>31</v>
       </c>
-      <c r="B35" s="72" t="inlineStr">
-        <is>
-          <t>1784313900011</t>
-        </is>
-      </c>
+      <c r="B35" s="72" t="n"/>
       <c r="C35" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -16801,11 +16677,7 @@
       <c r="A36" s="71" t="n">
         <v>32</v>
       </c>
-      <c r="B36" s="72" t="inlineStr">
-        <is>
-          <t>1784313900010</t>
-        </is>
-      </c>
+      <c r="B36" s="72" t="n"/>
       <c r="C36" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -16896,11 +16768,7 @@
       <c r="A37" s="71" t="n">
         <v>33</v>
       </c>
-      <c r="B37" s="72" t="inlineStr">
-        <is>
-          <t>1784313900018</t>
-        </is>
-      </c>
+      <c r="B37" s="72" t="n"/>
       <c r="C37" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -16991,11 +16859,7 @@
       <c r="A38" s="71" t="n">
         <v>34</v>
       </c>
-      <c r="B38" s="72" t="inlineStr">
-        <is>
-          <t>1784313900002</t>
-        </is>
-      </c>
+      <c r="B38" s="72" t="n"/>
       <c r="C38" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -17086,11 +16950,7 @@
       <c r="A39" s="71" t="n">
         <v>35</v>
       </c>
-      <c r="B39" s="72" t="inlineStr">
-        <is>
-          <t>1784313900048</t>
-        </is>
-      </c>
+      <c r="B39" s="72" t="n"/>
       <c r="C39" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -17181,11 +17041,7 @@
       <c r="A40" s="71" t="n">
         <v>36</v>
       </c>
-      <c r="B40" s="72" t="inlineStr">
-        <is>
-          <t>1784313900064</t>
-        </is>
-      </c>
+      <c r="B40" s="72" t="n"/>
       <c r="C40" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -17276,11 +17132,7 @@
       <c r="A41" s="71" t="n">
         <v>37</v>
       </c>
-      <c r="B41" s="72" t="inlineStr">
-        <is>
-          <t>1784313900015</t>
-        </is>
-      </c>
+      <c r="B41" s="72" t="n"/>
       <c r="C41" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -17371,11 +17223,7 @@
       <c r="A42" s="71" t="n">
         <v>38</v>
       </c>
-      <c r="B42" s="72" t="inlineStr">
-        <is>
-          <t>1784313900009</t>
-        </is>
-      </c>
+      <c r="B42" s="72" t="n"/>
       <c r="C42" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -17466,11 +17314,7 @@
       <c r="A43" s="71" t="n">
         <v>39</v>
       </c>
-      <c r="B43" s="72" t="inlineStr">
-        <is>
-          <t>1784313900021</t>
-        </is>
-      </c>
+      <c r="B43" s="72" t="n"/>
       <c r="C43" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -17561,11 +17405,7 @@
       <c r="A44" s="71" t="n">
         <v>40</v>
       </c>
-      <c r="B44" s="72" t="inlineStr">
-        <is>
-          <t>1784313900030</t>
-        </is>
-      </c>
+      <c r="B44" s="72" t="n"/>
       <c r="C44" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -17656,11 +17496,7 @@
       <c r="A45" s="71" t="n">
         <v>41</v>
       </c>
-      <c r="B45" s="72" t="inlineStr">
-        <is>
-          <t>1784313900026</t>
-        </is>
-      </c>
+      <c r="B45" s="72" t="n"/>
       <c r="C45" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -17751,11 +17587,7 @@
       <c r="A46" s="71" t="n">
         <v>42</v>
       </c>
-      <c r="B46" s="72" t="inlineStr">
-        <is>
-          <t>1784313900003</t>
-        </is>
-      </c>
+      <c r="B46" s="72" t="n"/>
       <c r="C46" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -17846,11 +17678,7 @@
       <c r="A47" s="71" t="n">
         <v>43</v>
       </c>
-      <c r="B47" s="72" t="inlineStr">
-        <is>
-          <t>1784313900062</t>
-        </is>
-      </c>
+      <c r="B47" s="72" t="n"/>
       <c r="C47" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -17941,11 +17769,7 @@
       <c r="A48" s="71" t="n">
         <v>44</v>
       </c>
-      <c r="B48" s="72" t="inlineStr">
-        <is>
-          <t>1784313900034</t>
-        </is>
-      </c>
+      <c r="B48" s="72" t="n"/>
       <c r="C48" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -18036,11 +17860,7 @@
       <c r="A49" s="71" t="n">
         <v>45</v>
       </c>
-      <c r="B49" s="72" t="inlineStr">
-        <is>
-          <t>1784313900025</t>
-        </is>
-      </c>
+      <c r="B49" s="72" t="n"/>
       <c r="C49" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -18131,11 +17951,7 @@
       <c r="A50" s="71" t="n">
         <v>46</v>
       </c>
-      <c r="B50" s="72" t="inlineStr">
-        <is>
-          <t>1784313900014</t>
-        </is>
-      </c>
+      <c r="B50" s="72" t="n"/>
       <c r="C50" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -18226,11 +18042,7 @@
       <c r="A51" s="71" t="n">
         <v>47</v>
       </c>
-      <c r="B51" s="72" t="inlineStr">
-        <is>
-          <t>1784313900033</t>
-        </is>
-      </c>
+      <c r="B51" s="72" t="n"/>
       <c r="C51" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -18321,11 +18133,7 @@
       <c r="A52" s="71" t="n">
         <v>48</v>
       </c>
-      <c r="B52" s="72" t="inlineStr">
-        <is>
-          <t>1784313900063</t>
-        </is>
-      </c>
+      <c r="B52" s="72" t="n"/>
       <c r="C52" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -18416,11 +18224,7 @@
       <c r="A53" s="71" t="n">
         <v>49</v>
       </c>
-      <c r="B53" s="72" t="inlineStr">
-        <is>
-          <t>1784313900016</t>
-        </is>
-      </c>
+      <c r="B53" s="72" t="n"/>
       <c r="C53" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -18511,11 +18315,7 @@
       <c r="A54" s="71" t="n">
         <v>50</v>
       </c>
-      <c r="B54" s="72" t="inlineStr">
-        <is>
-          <t>1784313900029</t>
-        </is>
-      </c>
+      <c r="B54" s="72" t="n"/>
       <c r="C54" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -18606,11 +18406,7 @@
       <c r="A55" s="71" t="n">
         <v>51</v>
       </c>
-      <c r="B55" s="72" t="inlineStr">
-        <is>
-          <t>1784313900020</t>
-        </is>
-      </c>
+      <c r="B55" s="72" t="n"/>
       <c r="C55" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -18701,11 +18497,7 @@
       <c r="A56" s="71" t="n">
         <v>52</v>
       </c>
-      <c r="B56" s="72" t="inlineStr">
-        <is>
-          <t>1784313900036</t>
-        </is>
-      </c>
+      <c r="B56" s="72" t="n"/>
       <c r="C56" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -18796,11 +18588,7 @@
       <c r="A57" s="71" t="n">
         <v>53</v>
       </c>
-      <c r="B57" s="72" t="inlineStr">
-        <is>
-          <t>1784313900006</t>
-        </is>
-      </c>
+      <c r="B57" s="72" t="n"/>
       <c r="C57" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -18891,11 +18679,7 @@
       <c r="A58" s="71" t="n">
         <v>54</v>
       </c>
-      <c r="B58" s="72" t="inlineStr">
-        <is>
-          <t>1784313900035</t>
-        </is>
-      </c>
+      <c r="B58" s="72" t="n"/>
       <c r="C58" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -18986,11 +18770,7 @@
       <c r="A59" s="71" t="n">
         <v>55</v>
       </c>
-      <c r="B59" s="72" t="inlineStr">
-        <is>
-          <t>1784313900008</t>
-        </is>
-      </c>
+      <c r="B59" s="72" t="n"/>
       <c r="C59" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -19081,11 +18861,7 @@
       <c r="A60" s="71" t="n">
         <v>56</v>
       </c>
-      <c r="B60" s="72" t="inlineStr">
-        <is>
-          <t>1784313900043</t>
-        </is>
-      </c>
+      <c r="B60" s="72" t="n"/>
       <c r="C60" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -19176,11 +18952,7 @@
       <c r="A61" s="71" t="n">
         <v>57</v>
       </c>
-      <c r="B61" s="72" t="inlineStr">
-        <is>
-          <t>1784313900058</t>
-        </is>
-      </c>
+      <c r="B61" s="72" t="n"/>
       <c r="C61" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -19271,11 +19043,7 @@
       <c r="A62" s="71" t="n">
         <v>58</v>
       </c>
-      <c r="B62" s="72" t="inlineStr">
-        <is>
-          <t>1784313900059</t>
-        </is>
-      </c>
+      <c r="B62" s="72" t="n"/>
       <c r="C62" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -19366,11 +19134,7 @@
       <c r="A63" s="71" t="n">
         <v>59</v>
       </c>
-      <c r="B63" s="72" t="inlineStr">
-        <is>
-          <t>1784313900053</t>
-        </is>
-      </c>
+      <c r="B63" s="72" t="n"/>
       <c r="C63" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -19461,11 +19225,7 @@
       <c r="A64" s="71" t="n">
         <v>60</v>
       </c>
-      <c r="B64" s="72" t="inlineStr">
-        <is>
-          <t>1784313900052</t>
-        </is>
-      </c>
+      <c r="B64" s="72" t="n"/>
       <c r="C64" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -19556,11 +19316,7 @@
       <c r="A65" s="71" t="n">
         <v>61</v>
       </c>
-      <c r="B65" s="72" t="inlineStr">
-        <is>
-          <t>1784313900060</t>
-        </is>
-      </c>
+      <c r="B65" s="72" t="n"/>
       <c r="C65" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -19651,11 +19407,7 @@
       <c r="A66" s="71" t="n">
         <v>62</v>
       </c>
-      <c r="B66" s="72" t="inlineStr">
-        <is>
-          <t>1784313900139</t>
-        </is>
-      </c>
+      <c r="B66" s="72" t="n"/>
       <c r="C66" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -19746,11 +19498,7 @@
       <c r="A67" s="71" t="n">
         <v>63</v>
       </c>
-      <c r="B67" s="72" t="inlineStr">
-        <is>
-          <t>1784313900078</t>
-        </is>
-      </c>
+      <c r="B67" s="72" t="n"/>
       <c r="C67" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -19841,11 +19589,7 @@
       <c r="A68" s="71" t="n">
         <v>64</v>
       </c>
-      <c r="B68" s="72" t="inlineStr">
-        <is>
-          <t>1784313900135</t>
-        </is>
-      </c>
+      <c r="B68" s="72" t="n"/>
       <c r="C68" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -19936,11 +19680,7 @@
       <c r="A69" s="71" t="n">
         <v>65</v>
       </c>
-      <c r="B69" s="72" t="inlineStr">
-        <is>
-          <t>1784313900004</t>
-        </is>
-      </c>
+      <c r="B69" s="72" t="n"/>
       <c r="C69" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -20031,11 +19771,7 @@
       <c r="A70" s="71" t="n">
         <v>66</v>
       </c>
-      <c r="B70" s="72" t="inlineStr">
-        <is>
-          <t>1784313901145</t>
-        </is>
-      </c>
+      <c r="B70" s="72" t="n"/>
       <c r="C70" t="inlineStr">
         <is>
           <t>wake</t>
@@ -20077,7 +19813,7 @@
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>/composition/layers/145/clips/1/connect</t>
+          <t>/composition/layers/145/clips/1/video/effects/transform/rotationz</t>
         </is>
       </c>
       <c r="M70" s="71" t="n">
@@ -20098,7 +19834,7 @@
       </c>
       <c r="U70" t="inlineStr">
         <is>
-          <t>/composition/layers/145/clips/1/connect</t>
+          <t>/composition/layers/145/clips/1/video/effects/transform/rotationz</t>
         </is>
       </c>
       <c r="X70" t="inlineStr">
@@ -20111,11 +19847,7 @@
       <c r="A71" s="71" t="n">
         <v>67</v>
       </c>
-      <c r="B71" s="72" t="inlineStr">
-        <is>
-          <t>1784313900145</t>
-        </is>
-      </c>
+      <c r="B71" s="72" t="n"/>
       <c r="C71" t="inlineStr">
         <is>
           <t>opacity</t>
@@ -20157,7 +19889,7 @@
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>/composition/layers/145/clips/1/video/opacity</t>
+          <t>/composition/layers/145/clips/1/video/effects/transform/rotationz</t>
         </is>
       </c>
       <c r="M71" s="71" t="n">
@@ -20187,7 +19919,7 @@
       </c>
       <c r="U71" t="inlineStr">
         <is>
-          <t>/composition/layers/145/clips/1/video/opacity</t>
+          <t>/composition/layers/145/clips/1/video/effects/transform/rotationz</t>
         </is>
       </c>
     </row>
@@ -20195,11 +19927,7 @@
       <c r="A72" s="71" t="n">
         <v>68</v>
       </c>
-      <c r="B72" s="72" t="inlineStr">
-        <is>
-          <t>1784313902145</t>
-        </is>
-      </c>
+      <c r="B72" s="72" t="n"/>
       <c r="C72" t="inlineStr">
         <is>
           <t>motion_rotation</t>
@@ -20279,11 +20007,7 @@
       <c r="A73" s="71" t="n">
         <v>69</v>
       </c>
-      <c r="B73" s="72" t="inlineStr">
-        <is>
-          <t>1784313901148</t>
-        </is>
-      </c>
+      <c r="B73" s="72" t="n"/>
       <c r="C73" t="inlineStr">
         <is>
           <t>wake</t>
@@ -20325,7 +20049,7 @@
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>/composition/layers/148/clips/1/connect</t>
+          <t>/composition/layers/148/clips/1/video/effects/transform/rotationz</t>
         </is>
       </c>
       <c r="M73" s="71" t="n">
@@ -20346,7 +20070,7 @@
       </c>
       <c r="U73" t="inlineStr">
         <is>
-          <t>/composition/layers/148/clips/1/connect</t>
+          <t>/composition/layers/148/clips/1/video/effects/transform/rotationz</t>
         </is>
       </c>
       <c r="X73" t="inlineStr">
@@ -20359,11 +20083,7 @@
       <c r="A74" s="71" t="n">
         <v>70</v>
       </c>
-      <c r="B74" s="72" t="inlineStr">
-        <is>
-          <t>1784313900148</t>
-        </is>
-      </c>
+      <c r="B74" s="72" t="n"/>
       <c r="C74" t="inlineStr">
         <is>
           <t>tempo_motion</t>
@@ -20439,11 +20159,7 @@
       <c r="A75" s="71" t="n">
         <v>71</v>
       </c>
-      <c r="B75" s="72" t="inlineStr">
-        <is>
-          <t>1784313900067</t>
-        </is>
-      </c>
+      <c r="B75" s="72" t="n"/>
       <c r="C75" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -20534,11 +20250,7 @@
       <c r="A76" s="71" t="n">
         <v>72</v>
       </c>
-      <c r="B76" s="72" t="inlineStr">
-        <is>
-          <t>1784313901094</t>
-        </is>
-      </c>
+      <c r="B76" s="72" t="n"/>
       <c r="C76" t="inlineStr">
         <is>
           <t>wake</t>
@@ -20606,7 +20318,7 @@
       </c>
       <c r="X76" t="inlineStr">
         <is>
-          <t>Disconnected=1</t>
+          <t>Connected=1; Disconnected=1</t>
         </is>
       </c>
     </row>
@@ -20614,11 +20326,7 @@
       <c r="A77" s="71" t="n">
         <v>73</v>
       </c>
-      <c r="B77" s="72" t="inlineStr">
-        <is>
-          <t>1784313900094</t>
-        </is>
-      </c>
+      <c r="B77" s="72" t="n"/>
       <c r="C77" t="inlineStr">
         <is>
           <t>opacity</t>
@@ -20660,7 +20368,7 @@
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>/composition/layers/94/clips/1/video/opacity</t>
+          <t>/composition/layers/94/clips/1/connect</t>
         </is>
       </c>
       <c r="M77" s="71" t="n">
@@ -20690,7 +20398,12 @@
       </c>
       <c r="U77" t="inlineStr">
         <is>
-          <t>/composition/layers/94/clips/1/video/opacity</t>
+          <t>/composition/layers/94/clips/1/connect</t>
+        </is>
+      </c>
+      <c r="X77" t="inlineStr">
+        <is>
+          <t>Connected=1; Disconnected=1</t>
         </is>
       </c>
     </row>
@@ -20698,11 +20411,7 @@
       <c r="A78" s="71" t="n">
         <v>74</v>
       </c>
-      <c r="B78" s="72" t="inlineStr">
-        <is>
-          <t>1784313902094</t>
-        </is>
-      </c>
+      <c r="B78" s="72" t="n"/>
       <c r="C78" t="inlineStr">
         <is>
           <t>motion_y</t>
@@ -20744,7 +20453,7 @@
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>/composition/layers/94/clips/1/video/effects/transform/positiony</t>
+          <t>/composition/layers/94/clips/1/connect</t>
         </is>
       </c>
       <c r="M78" s="71" t="n">
@@ -20774,7 +20483,12 @@
       </c>
       <c r="U78" t="inlineStr">
         <is>
-          <t>/composition/layers/94/clips/1/video/effects/transform/positiony</t>
+          <t>/composition/layers/94/clips/1/connect</t>
+        </is>
+      </c>
+      <c r="X78" t="inlineStr">
+        <is>
+          <t>Connected=1; Disconnected=1</t>
         </is>
       </c>
     </row>
@@ -20782,11 +20496,7 @@
       <c r="A79" s="71" t="n">
         <v>75</v>
       </c>
-      <c r="B79" s="72" t="inlineStr">
-        <is>
-          <t>1784313900070</t>
-        </is>
-      </c>
+      <c r="B79" s="72" t="n"/>
       <c r="C79" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -20877,11 +20587,7 @@
       <c r="A80" s="71" t="n">
         <v>76</v>
       </c>
-      <c r="B80" s="72" t="inlineStr">
-        <is>
-          <t>1784313900147</t>
-        </is>
-      </c>
+      <c r="B80" s="72" t="n"/>
       <c r="C80" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -20972,11 +20678,7 @@
       <c r="A81" s="71" t="n">
         <v>77</v>
       </c>
-      <c r="B81" s="72" t="inlineStr">
-        <is>
-          <t>1784313900140</t>
-        </is>
-      </c>
+      <c r="B81" s="72" t="n"/>
       <c r="C81" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -21067,11 +20769,7 @@
       <c r="A82" s="71" t="n">
         <v>78</v>
       </c>
-      <c r="B82" s="72" t="inlineStr">
-        <is>
-          <t>1784313900082</t>
-        </is>
-      </c>
+      <c r="B82" s="72" t="n"/>
       <c r="C82" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -21162,11 +20860,7 @@
       <c r="A83" s="71" t="n">
         <v>79</v>
       </c>
-      <c r="B83" s="72" t="inlineStr">
-        <is>
-          <t>1784313900090</t>
-        </is>
-      </c>
+      <c r="B83" s="72" t="n"/>
       <c r="C83" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -21249,7 +20943,7 @@
       </c>
       <c r="X83" t="inlineStr">
         <is>
-          <t>Connected=0.070866141732283463583; Connected &amp; previewing=0.070866141732283463583; Disconnected=0; Empty=0; Off=0; Previewing=0</t>
+          <t>Connected=1.0; Connected &amp; previewing=1.0; Disconnected=1.0; Empty=0; Off=0; Previewing=0</t>
         </is>
       </c>
     </row>
@@ -21257,11 +20951,7 @@
       <c r="A84" s="71" t="n">
         <v>80</v>
       </c>
-      <c r="B84" s="72" t="inlineStr">
-        <is>
-          <t>1784313900137</t>
-        </is>
-      </c>
+      <c r="B84" s="72" t="n"/>
       <c r="C84" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -21352,11 +21042,7 @@
       <c r="A85" s="71" t="n">
         <v>81</v>
       </c>
-      <c r="B85" s="72" t="inlineStr">
-        <is>
-          <t>1784313900138</t>
-        </is>
-      </c>
+      <c r="B85" s="72" t="n"/>
       <c r="C85" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -21447,11 +21133,7 @@
       <c r="A86" s="71" t="n">
         <v>82</v>
       </c>
-      <c r="B86" s="72" t="inlineStr">
-        <is>
-          <t>1784313900072</t>
-        </is>
-      </c>
+      <c r="B86" s="72" t="n"/>
       <c r="C86" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -21542,11 +21224,7 @@
       <c r="A87" s="71" t="n">
         <v>83</v>
       </c>
-      <c r="B87" s="72" t="inlineStr">
-        <is>
-          <t>1784313900142</t>
-        </is>
-      </c>
+      <c r="B87" s="72" t="n"/>
       <c r="C87" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -21637,11 +21315,7 @@
       <c r="A88" s="71" t="n">
         <v>84</v>
       </c>
-      <c r="B88" s="72" t="inlineStr">
-        <is>
-          <t>1784313900141</t>
-        </is>
-      </c>
+      <c r="B88" s="72" t="n"/>
       <c r="C88" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -21732,11 +21406,7 @@
       <c r="A89" s="71" t="n">
         <v>85</v>
       </c>
-      <c r="B89" s="72" t="inlineStr">
-        <is>
-          <t>1784313900092</t>
-        </is>
-      </c>
+      <c r="B89" s="72" t="n"/>
       <c r="C89" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -21819,7 +21489,7 @@
       </c>
       <c r="X89" t="inlineStr">
         <is>
-          <t>Connected=0.070866141732283463583; Connected &amp; previewing=0.070866141732283463583; Disconnected=0; Empty=0; Off=0; Previewing=0</t>
+          <t>Connected=1.0; Connected &amp; previewing=1.0; Disconnected=1.0; Empty=0; Off=0; Previewing=0</t>
         </is>
       </c>
     </row>
@@ -21827,11 +21497,7 @@
       <c r="A90" s="71" t="n">
         <v>86</v>
       </c>
-      <c r="B90" s="72" t="inlineStr">
-        <is>
-          <t>1784313900071</t>
-        </is>
-      </c>
+      <c r="B90" s="72" t="n"/>
       <c r="C90" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -21922,11 +21588,7 @@
       <c r="A91" s="71" t="n">
         <v>87</v>
       </c>
-      <c r="B91" s="72" t="inlineStr">
-        <is>
-          <t>1784313900038</t>
-        </is>
-      </c>
+      <c r="B91" s="72" t="n"/>
       <c r="C91" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -22017,11 +21679,7 @@
       <c r="A92" s="71" t="n">
         <v>88</v>
       </c>
-      <c r="B92" s="72" t="inlineStr">
-        <is>
-          <t>1784313901144</t>
-        </is>
-      </c>
+      <c r="B92" s="72" t="n"/>
       <c r="C92" t="inlineStr">
         <is>
           <t>wake</t>
@@ -22063,7 +21721,7 @@
       </c>
       <c r="L92" t="inlineStr">
         <is>
-          <t>/composition/layers/144/clips/1/connect</t>
+          <t>/composition/layers/144/clips/1/video/opacity</t>
         </is>
       </c>
       <c r="M92" s="71" t="n">
@@ -22084,7 +21742,7 @@
       </c>
       <c r="U92" t="inlineStr">
         <is>
-          <t>/composition/layers/144/clips/1/connect</t>
+          <t>/composition/layers/144/clips/1/video/opacity</t>
         </is>
       </c>
       <c r="X92" t="inlineStr">
@@ -22097,11 +21755,7 @@
       <c r="A93" s="71" t="n">
         <v>89</v>
       </c>
-      <c r="B93" s="72" t="inlineStr">
-        <is>
-          <t>1784313900144</t>
-        </is>
-      </c>
+      <c r="B93" s="72" t="n"/>
       <c r="C93" t="inlineStr">
         <is>
           <t>opacity</t>
@@ -22181,11 +21835,7 @@
       <c r="A94" s="71" t="n">
         <v>90</v>
       </c>
-      <c r="B94" s="72" t="inlineStr">
-        <is>
-          <t>1784313902144</t>
-        </is>
-      </c>
+      <c r="B94" s="72" t="n"/>
       <c r="C94" t="inlineStr">
         <is>
           <t>motion_x</t>
@@ -22227,7 +21877,7 @@
       </c>
       <c r="L94" t="inlineStr">
         <is>
-          <t>/composition/layers/144/clips/1/video/effects/transform/positionx</t>
+          <t>/composition/layers/144/clips/1/video/opacity</t>
         </is>
       </c>
       <c r="M94" s="71" t="n">
@@ -22257,7 +21907,7 @@
       </c>
       <c r="U94" t="inlineStr">
         <is>
-          <t>/composition/layers/144/clips/1/video/effects/transform/positionx</t>
+          <t>/composition/layers/144/clips/1/video/opacity</t>
         </is>
       </c>
     </row>
@@ -22265,11 +21915,7 @@
       <c r="A95" s="71" t="n">
         <v>91</v>
       </c>
-      <c r="B95" s="72" t="inlineStr">
-        <is>
-          <t>1784313901143</t>
-        </is>
-      </c>
+      <c r="B95" s="72" t="n"/>
       <c r="C95" t="inlineStr">
         <is>
           <t>wake</t>
@@ -22337,7 +21983,7 @@
       </c>
       <c r="X95" t="inlineStr">
         <is>
-          <t>Disconnected=1</t>
+          <t>Connected=1; Disconnected=1</t>
         </is>
       </c>
     </row>
@@ -22345,11 +21991,7 @@
       <c r="A96" s="71" t="n">
         <v>92</v>
       </c>
-      <c r="B96" s="72" t="inlineStr">
-        <is>
-          <t>1784313900143</t>
-        </is>
-      </c>
+      <c r="B96" s="72" t="n"/>
       <c r="C96" t="inlineStr">
         <is>
           <t>opacity</t>
@@ -22391,7 +22033,7 @@
       </c>
       <c r="L96" t="inlineStr">
         <is>
-          <t>/composition/layers/143/clips/1/video/opacity</t>
+          <t>/composition/layers/143/clips/1/connect</t>
         </is>
       </c>
       <c r="M96" s="71" t="n">
@@ -22421,7 +22063,12 @@
       </c>
       <c r="U96" t="inlineStr">
         <is>
-          <t>/composition/layers/143/clips/1/video/opacity</t>
+          <t>/composition/layers/143/clips/1/connect</t>
+        </is>
+      </c>
+      <c r="X96" t="inlineStr">
+        <is>
+          <t>Connected=1; Disconnected=1</t>
         </is>
       </c>
     </row>
@@ -22429,11 +22076,7 @@
       <c r="A97" s="71" t="n">
         <v>93</v>
       </c>
-      <c r="B97" s="72" t="inlineStr">
-        <is>
-          <t>1784313902143</t>
-        </is>
-      </c>
+      <c r="B97" s="72" t="n"/>
       <c r="C97" t="inlineStr">
         <is>
           <t>motion_y</t>
@@ -22475,7 +22118,7 @@
       </c>
       <c r="L97" t="inlineStr">
         <is>
-          <t>/composition/layers/143/clips/1/video/effects/transform/positiony</t>
+          <t>/composition/layers/143/clips/1/connect</t>
         </is>
       </c>
       <c r="M97" s="71" t="n">
@@ -22505,7 +22148,12 @@
       </c>
       <c r="U97" t="inlineStr">
         <is>
-          <t>/composition/layers/143/clips/1/video/effects/transform/positiony</t>
+          <t>/composition/layers/143/clips/1/connect</t>
+        </is>
+      </c>
+      <c r="X97" t="inlineStr">
+        <is>
+          <t>Connected=1; Disconnected=1</t>
         </is>
       </c>
     </row>
@@ -22513,11 +22161,7 @@
       <c r="A98" s="71" t="n">
         <v>94</v>
       </c>
-      <c r="B98" s="72" t="inlineStr">
-        <is>
-          <t>1784313900080</t>
-        </is>
-      </c>
+      <c r="B98" s="72" t="n"/>
       <c r="C98" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -22608,11 +22252,7 @@
       <c r="A99" s="71" t="n">
         <v>95</v>
       </c>
-      <c r="B99" s="72" t="inlineStr">
-        <is>
-          <t>1784313900028</t>
-        </is>
-      </c>
+      <c r="B99" s="72" t="n"/>
       <c r="C99" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -22703,11 +22343,7 @@
       <c r="A100" s="71" t="n">
         <v>96</v>
       </c>
-      <c r="B100" s="72" t="inlineStr">
-        <is>
-          <t>1784313900079</t>
-        </is>
-      </c>
+      <c r="B100" s="72" t="n"/>
       <c r="C100" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -22798,11 +22434,7 @@
       <c r="A101" s="71" t="n">
         <v>97</v>
       </c>
-      <c r="B101" s="72" t="inlineStr">
-        <is>
-          <t>1784313900069</t>
-        </is>
-      </c>
+      <c r="B101" s="72" t="n"/>
       <c r="C101" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -22893,11 +22525,7 @@
       <c r="A102" s="71" t="n">
         <v>98</v>
       </c>
-      <c r="B102" s="72" t="inlineStr">
-        <is>
-          <t>1784313900146</t>
-        </is>
-      </c>
+      <c r="B102" s="72" t="n"/>
       <c r="C102" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -22988,11 +22616,7 @@
       <c r="A103" s="71" t="n">
         <v>99</v>
       </c>
-      <c r="B103" s="72" t="inlineStr">
-        <is>
-          <t>1784313900077</t>
-        </is>
-      </c>
+      <c r="B103" s="72" t="n"/>
       <c r="C103" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -23083,11 +22707,7 @@
       <c r="A104" s="71" t="n">
         <v>100</v>
       </c>
-      <c r="B104" s="72" t="inlineStr">
-        <is>
-          <t>1784313900073</t>
-        </is>
-      </c>
+      <c r="B104" s="72" t="n"/>
       <c r="C104" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -23178,11 +22798,7 @@
       <c r="A105" s="71" t="n">
         <v>101</v>
       </c>
-      <c r="B105" s="72" t="inlineStr">
-        <is>
-          <t>1784313900087</t>
-        </is>
-      </c>
+      <c r="B105" s="72" t="n"/>
       <c r="C105" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -23265,7 +22881,7 @@
       </c>
       <c r="X105" t="inlineStr">
         <is>
-          <t>Connected=0.070866141732283463583; Connected &amp; previewing=0.070866141732283463583; Disconnected=0; Empty=0; Off=0; Previewing=0</t>
+          <t>Connected=1.0; Connected &amp; previewing=1.0; Disconnected=1.0; Empty=0; Off=0; Previewing=0</t>
         </is>
       </c>
     </row>
@@ -23273,11 +22889,7 @@
       <c r="A106" s="71" t="n">
         <v>102</v>
       </c>
-      <c r="B106" s="72" t="inlineStr">
-        <is>
-          <t>1784313900136</t>
-        </is>
-      </c>
+      <c r="B106" s="72" t="n"/>
       <c r="C106" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -23368,11 +22980,7 @@
       <c r="A107" s="71" t="n">
         <v>103</v>
       </c>
-      <c r="B107" s="72" t="inlineStr">
-        <is>
-          <t>1784313900091</t>
-        </is>
-      </c>
+      <c r="B107" s="72" t="n"/>
       <c r="C107" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -23455,7 +23063,7 @@
       </c>
       <c r="X107" t="inlineStr">
         <is>
-          <t>Connected=0.070866141732283463583; Connected &amp; previewing=0.070866141732283463583; Disconnected=0; Empty=0; Off=0; Previewing=0</t>
+          <t>Connected=1.0; Connected &amp; previewing=1.0; Disconnected=1.0; Empty=0; Off=0; Previewing=0</t>
         </is>
       </c>
     </row>
@@ -23463,11 +23071,7 @@
       <c r="A108" s="71" t="n">
         <v>104</v>
       </c>
-      <c r="B108" s="72" t="inlineStr">
-        <is>
-          <t>1784313900085</t>
-        </is>
-      </c>
+      <c r="B108" s="72" t="n"/>
       <c r="C108" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -23558,11 +23162,7 @@
       <c r="A109" s="71" t="n">
         <v>105</v>
       </c>
-      <c r="B109" s="72" t="inlineStr">
-        <is>
-          <t>1784313901099</t>
-        </is>
-      </c>
+      <c r="B109" s="72" t="n"/>
       <c r="C109" t="inlineStr">
         <is>
           <t>wake</t>
@@ -23604,7 +23204,7 @@
       </c>
       <c r="L109" t="inlineStr">
         <is>
-          <t>/composition/layers/99/clips/1/connect</t>
+          <t>/composition/layers/99/clips/1/video/effects/transform/positiony</t>
         </is>
       </c>
       <c r="M109" s="71" t="n">
@@ -23625,7 +23225,7 @@
       </c>
       <c r="U109" t="inlineStr">
         <is>
-          <t>/composition/layers/99/clips/1/connect</t>
+          <t>/composition/layers/99/clips/1/video/effects/transform/positiony</t>
         </is>
       </c>
       <c r="X109" t="inlineStr">
@@ -23638,11 +23238,7 @@
       <c r="A110" s="71" t="n">
         <v>106</v>
       </c>
-      <c r="B110" s="72" t="inlineStr">
-        <is>
-          <t>1784313900099</t>
-        </is>
-      </c>
+      <c r="B110" s="72" t="n"/>
       <c r="C110" t="inlineStr">
         <is>
           <t>opacity</t>
@@ -23684,7 +23280,7 @@
       </c>
       <c r="L110" t="inlineStr">
         <is>
-          <t>/composition/layers/99/clips/1/video/opacity</t>
+          <t>/composition/layers/99/clips/1/video/effects/transform/positiony</t>
         </is>
       </c>
       <c r="M110" s="71" t="n">
@@ -23714,7 +23310,7 @@
       </c>
       <c r="U110" t="inlineStr">
         <is>
-          <t>/composition/layers/99/clips/1/video/opacity</t>
+          <t>/composition/layers/99/clips/1/video/effects/transform/positiony</t>
         </is>
       </c>
     </row>
@@ -23722,11 +23318,7 @@
       <c r="A111" s="71" t="n">
         <v>107</v>
       </c>
-      <c r="B111" s="72" t="inlineStr">
-        <is>
-          <t>1784313902099</t>
-        </is>
-      </c>
+      <c r="B111" s="72" t="n"/>
       <c r="C111" t="inlineStr">
         <is>
           <t>motion_y</t>
@@ -23806,11 +23398,7 @@
       <c r="A112" s="71" t="n">
         <v>108</v>
       </c>
-      <c r="B112" s="72" t="inlineStr">
-        <is>
-          <t>1784313900075</t>
-        </is>
-      </c>
+      <c r="B112" s="72" t="n"/>
       <c r="C112" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -23901,11 +23489,7 @@
       <c r="A113" s="71" t="n">
         <v>109</v>
       </c>
-      <c r="B113" s="72" t="inlineStr">
-        <is>
-          <t>1784313901109</t>
-        </is>
-      </c>
+      <c r="B113" s="72" t="n"/>
       <c r="C113" t="inlineStr">
         <is>
           <t>wake</t>
@@ -23973,7 +23557,7 @@
       </c>
       <c r="X113" t="inlineStr">
         <is>
-          <t>Disconnected=1</t>
+          <t>Connected=1; Disconnected=1</t>
         </is>
       </c>
     </row>
@@ -23981,11 +23565,7 @@
       <c r="A114" s="71" t="n">
         <v>110</v>
       </c>
-      <c r="B114" s="72" t="inlineStr">
-        <is>
-          <t>1784313900109</t>
-        </is>
-      </c>
+      <c r="B114" s="72" t="n"/>
       <c r="C114" t="inlineStr">
         <is>
           <t>opacity</t>
@@ -24027,7 +23607,7 @@
       </c>
       <c r="L114" t="inlineStr">
         <is>
-          <t>/composition/layers/109/clips/1/video/opacity</t>
+          <t>/composition/layers/109/clips/1/connect</t>
         </is>
       </c>
       <c r="M114" s="71" t="n">
@@ -24057,7 +23637,12 @@
       </c>
       <c r="U114" t="inlineStr">
         <is>
-          <t>/composition/layers/109/clips/1/video/opacity</t>
+          <t>/composition/layers/109/clips/1/connect</t>
+        </is>
+      </c>
+      <c r="X114" t="inlineStr">
+        <is>
+          <t>Connected=1; Disconnected=1</t>
         </is>
       </c>
     </row>
@@ -24065,11 +23650,7 @@
       <c r="A115" s="71" t="n">
         <v>111</v>
       </c>
-      <c r="B115" s="72" t="inlineStr">
-        <is>
-          <t>1784313902109</t>
-        </is>
-      </c>
+      <c r="B115" s="72" t="n"/>
       <c r="C115" t="inlineStr">
         <is>
           <t>motion_rotation</t>
@@ -24111,7 +23692,7 @@
       </c>
       <c r="L115" t="inlineStr">
         <is>
-          <t>/composition/layers/109/clips/1/video/effects/transform/rotationz</t>
+          <t>/composition/layers/109/clips/1/connect</t>
         </is>
       </c>
       <c r="M115" s="71" t="n">
@@ -24141,7 +23722,12 @@
       </c>
       <c r="U115" t="inlineStr">
         <is>
-          <t>/composition/layers/109/clips/1/video/effects/transform/rotationz</t>
+          <t>/composition/layers/109/clips/1/connect</t>
+        </is>
+      </c>
+      <c r="X115" t="inlineStr">
+        <is>
+          <t>Connected=1; Disconnected=1</t>
         </is>
       </c>
     </row>
@@ -24149,11 +23735,7 @@
       <c r="A116" s="71" t="n">
         <v>112</v>
       </c>
-      <c r="B116" s="72" t="inlineStr">
-        <is>
-          <t>1784313900120</t>
-        </is>
-      </c>
+      <c r="B116" s="72" t="n"/>
       <c r="C116" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -24244,11 +23826,7 @@
       <c r="A117" s="71" t="n">
         <v>113</v>
       </c>
-      <c r="B117" s="72" t="inlineStr">
-        <is>
-          <t>1784313901106</t>
-        </is>
-      </c>
+      <c r="B117" s="72" t="n"/>
       <c r="C117" t="inlineStr">
         <is>
           <t>wake</t>
@@ -24290,7 +23868,7 @@
       </c>
       <c r="L117" t="inlineStr">
         <is>
-          <t>/composition/layers/106/clips/1/connect</t>
+          <t>/composition/layers/106/clips/1/video/effects/transform/rotationz</t>
         </is>
       </c>
       <c r="M117" s="71" t="n">
@@ -24311,7 +23889,7 @@
       </c>
       <c r="U117" t="inlineStr">
         <is>
-          <t>/composition/layers/106/clips/1/connect</t>
+          <t>/composition/layers/106/clips/1/video/effects/transform/rotationz</t>
         </is>
       </c>
       <c r="X117" t="inlineStr">
@@ -24324,11 +23902,7 @@
       <c r="A118" s="71" t="n">
         <v>114</v>
       </c>
-      <c r="B118" s="72" t="inlineStr">
-        <is>
-          <t>1784313900106</t>
-        </is>
-      </c>
+      <c r="B118" s="72" t="n"/>
       <c r="C118" t="inlineStr">
         <is>
           <t>opacity</t>
@@ -24370,7 +23944,7 @@
       </c>
       <c r="L118" t="inlineStr">
         <is>
-          <t>/composition/layers/106/clips/1/video/opacity</t>
+          <t>/composition/layers/106/clips/1/video/effects/transform/rotationz</t>
         </is>
       </c>
       <c r="M118" s="71" t="n">
@@ -24400,7 +23974,7 @@
       </c>
       <c r="U118" t="inlineStr">
         <is>
-          <t>/composition/layers/106/clips/1/video/opacity</t>
+          <t>/composition/layers/106/clips/1/video/effects/transform/rotationz</t>
         </is>
       </c>
     </row>
@@ -24408,11 +23982,7 @@
       <c r="A119" s="71" t="n">
         <v>115</v>
       </c>
-      <c r="B119" s="72" t="inlineStr">
-        <is>
-          <t>1784313902106</t>
-        </is>
-      </c>
+      <c r="B119" s="72" t="n"/>
       <c r="C119" t="inlineStr">
         <is>
           <t>motion_rotation</t>
@@ -24492,11 +24062,7 @@
       <c r="A120" s="71" t="n">
         <v>116</v>
       </c>
-      <c r="B120" s="72" t="inlineStr">
-        <is>
-          <t>1784313900066</t>
-        </is>
-      </c>
+      <c r="B120" s="72" t="n"/>
       <c r="C120" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -24587,11 +24153,7 @@
       <c r="A121" s="71" t="n">
         <v>117</v>
       </c>
-      <c r="B121" s="72" t="inlineStr">
-        <is>
-          <t>1784313900083</t>
-        </is>
-      </c>
+      <c r="B121" s="72" t="n"/>
       <c r="C121" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -24682,11 +24244,7 @@
       <c r="A122" s="71" t="n">
         <v>118</v>
       </c>
-      <c r="B122" s="72" t="inlineStr">
-        <is>
-          <t>1784313901114</t>
-        </is>
-      </c>
+      <c r="B122" s="72" t="n"/>
       <c r="C122" t="inlineStr">
         <is>
           <t>wake</t>
@@ -24728,7 +24286,7 @@
       </c>
       <c r="L122" t="inlineStr">
         <is>
-          <t>/composition/layers/114/clips/1/connect</t>
+          <t>/composition/layers/114/clips/1/video/opacity</t>
         </is>
       </c>
       <c r="M122" s="71" t="n">
@@ -24749,7 +24307,7 @@
       </c>
       <c r="U122" t="inlineStr">
         <is>
-          <t>/composition/layers/114/clips/1/connect</t>
+          <t>/composition/layers/114/clips/1/video/opacity</t>
         </is>
       </c>
       <c r="X122" t="inlineStr">
@@ -24762,11 +24320,7 @@
       <c r="A123" s="71" t="n">
         <v>119</v>
       </c>
-      <c r="B123" s="72" t="inlineStr">
-        <is>
-          <t>1784313900114</t>
-        </is>
-      </c>
+      <c r="B123" s="72" t="n"/>
       <c r="C123" t="inlineStr">
         <is>
           <t>opacity</t>
@@ -24846,11 +24400,7 @@
       <c r="A124" s="71" t="n">
         <v>120</v>
       </c>
-      <c r="B124" s="72" t="inlineStr">
-        <is>
-          <t>1784313902114</t>
-        </is>
-      </c>
+      <c r="B124" s="72" t="n"/>
       <c r="C124" t="inlineStr">
         <is>
           <t>motion_rotation</t>
@@ -24892,7 +24442,7 @@
       </c>
       <c r="L124" t="inlineStr">
         <is>
-          <t>/composition/layers/114/clips/1/video/effects/transform/rotationz</t>
+          <t>/composition/layers/114/clips/1/video/opacity</t>
         </is>
       </c>
       <c r="M124" s="71" t="n">
@@ -24922,7 +24472,7 @@
       </c>
       <c r="U124" t="inlineStr">
         <is>
-          <t>/composition/layers/114/clips/1/video/effects/transform/rotationz</t>
+          <t>/composition/layers/114/clips/1/video/opacity</t>
         </is>
       </c>
     </row>
@@ -24930,11 +24480,7 @@
       <c r="A125" s="71" t="n">
         <v>121</v>
       </c>
-      <c r="B125" s="72" t="inlineStr">
-        <is>
-          <t>1784313900122</t>
-        </is>
-      </c>
+      <c r="B125" s="72" t="n"/>
       <c r="C125" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -25025,11 +24571,7 @@
       <c r="A126" s="71" t="n">
         <v>122</v>
       </c>
-      <c r="B126" s="72" t="inlineStr">
-        <is>
-          <t>1784313900086</t>
-        </is>
-      </c>
+      <c r="B126" s="72" t="n"/>
       <c r="C126" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -25112,7 +24654,7 @@
       </c>
       <c r="X126" t="inlineStr">
         <is>
-          <t>Connected=0.070866141732283463583; Connected &amp; previewing=0.070866141732283463583; Disconnected=0; Empty=0; Off=0; Previewing=0</t>
+          <t>Connected=1.0; Connected &amp; previewing=1.0; Disconnected=1.0; Empty=0; Off=0; Previewing=0</t>
         </is>
       </c>
     </row>
@@ -25120,11 +24662,7 @@
       <c r="A127" s="71" t="n">
         <v>123</v>
       </c>
-      <c r="B127" s="72" t="inlineStr">
-        <is>
-          <t>1784313901113</t>
-        </is>
-      </c>
+      <c r="B127" s="72" t="n"/>
       <c r="C127" t="inlineStr">
         <is>
           <t>wake</t>
@@ -25192,7 +24730,7 @@
       </c>
       <c r="X127" t="inlineStr">
         <is>
-          <t>Disconnected=1</t>
+          <t>Connected=1; Disconnected=1</t>
         </is>
       </c>
     </row>
@@ -25200,11 +24738,7 @@
       <c r="A128" s="71" t="n">
         <v>124</v>
       </c>
-      <c r="B128" s="72" t="inlineStr">
-        <is>
-          <t>1784313900113</t>
-        </is>
-      </c>
+      <c r="B128" s="72" t="n"/>
       <c r="C128" t="inlineStr">
         <is>
           <t>opacity</t>
@@ -25246,7 +24780,7 @@
       </c>
       <c r="L128" t="inlineStr">
         <is>
-          <t>/composition/layers/113/clips/1/video/opacity</t>
+          <t>/composition/layers/113/clips/1/connect</t>
         </is>
       </c>
       <c r="M128" s="71" t="n">
@@ -25276,7 +24810,12 @@
       </c>
       <c r="U128" t="inlineStr">
         <is>
-          <t>/composition/layers/113/clips/1/video/opacity</t>
+          <t>/composition/layers/113/clips/1/connect</t>
+        </is>
+      </c>
+      <c r="X128" t="inlineStr">
+        <is>
+          <t>Connected=1; Disconnected=1</t>
         </is>
       </c>
     </row>
@@ -25284,11 +24823,7 @@
       <c r="A129" s="71" t="n">
         <v>125</v>
       </c>
-      <c r="B129" s="72" t="inlineStr">
-        <is>
-          <t>1784313902113</t>
-        </is>
-      </c>
+      <c r="B129" s="72" t="n"/>
       <c r="C129" t="inlineStr">
         <is>
           <t>motion_rotation</t>
@@ -25330,7 +24865,7 @@
       </c>
       <c r="L129" t="inlineStr">
         <is>
-          <t>/composition/layers/113/clips/1/video/effects/transform/rotationz</t>
+          <t>/composition/layers/113/clips/1/connect</t>
         </is>
       </c>
       <c r="M129" s="71" t="n">
@@ -25360,7 +24895,12 @@
       </c>
       <c r="U129" t="inlineStr">
         <is>
-          <t>/composition/layers/113/clips/1/video/effects/transform/rotationz</t>
+          <t>/composition/layers/113/clips/1/connect</t>
+        </is>
+      </c>
+      <c r="X129" t="inlineStr">
+        <is>
+          <t>Connected=1; Disconnected=1</t>
         </is>
       </c>
     </row>
@@ -25368,11 +24908,7 @@
       <c r="A130" s="71" t="n">
         <v>126</v>
       </c>
-      <c r="B130" s="72" t="inlineStr">
-        <is>
-          <t>1784313901104</t>
-        </is>
-      </c>
+      <c r="B130" s="72" t="n"/>
       <c r="C130" t="inlineStr">
         <is>
           <t>wake</t>
@@ -25414,7 +24950,7 @@
       </c>
       <c r="L130" t="inlineStr">
         <is>
-          <t>/composition/layers/104/clips/1/connect</t>
+          <t>/composition/layers/104/clips/1/video/opacity</t>
         </is>
       </c>
       <c r="M130" s="71" t="n">
@@ -25435,7 +24971,7 @@
       </c>
       <c r="U130" t="inlineStr">
         <is>
-          <t>/composition/layers/104/clips/1/connect</t>
+          <t>/composition/layers/104/clips/1/video/opacity</t>
         </is>
       </c>
       <c r="X130" t="inlineStr">
@@ -25448,11 +24984,7 @@
       <c r="A131" s="71" t="n">
         <v>127</v>
       </c>
-      <c r="B131" s="72" t="inlineStr">
-        <is>
-          <t>1784313900104</t>
-        </is>
-      </c>
+      <c r="B131" s="72" t="n"/>
       <c r="C131" t="inlineStr">
         <is>
           <t>opacity</t>
@@ -25532,11 +25064,7 @@
       <c r="A132" s="71" t="n">
         <v>128</v>
       </c>
-      <c r="B132" s="72" t="inlineStr">
-        <is>
-          <t>1784313902104</t>
-        </is>
-      </c>
+      <c r="B132" s="72" t="n"/>
       <c r="C132" t="inlineStr">
         <is>
           <t>motion_rotation</t>
@@ -25578,7 +25106,7 @@
       </c>
       <c r="L132" t="inlineStr">
         <is>
-          <t>/composition/layers/104/clips/1/video/effects/transform/rotationz</t>
+          <t>/composition/layers/104/clips/1/video/opacity</t>
         </is>
       </c>
       <c r="M132" s="71" t="n">
@@ -25608,7 +25136,7 @@
       </c>
       <c r="U132" t="inlineStr">
         <is>
-          <t>/composition/layers/104/clips/1/video/effects/transform/rotationz</t>
+          <t>/composition/layers/104/clips/1/video/opacity</t>
         </is>
       </c>
     </row>
@@ -25616,11 +25144,7 @@
       <c r="A133" s="71" t="n">
         <v>129</v>
       </c>
-      <c r="B133" s="72" t="inlineStr">
-        <is>
-          <t>1784313900065</t>
-        </is>
-      </c>
+      <c r="B133" s="72" t="n"/>
       <c r="C133" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -25711,11 +25235,7 @@
       <c r="A134" s="71" t="n">
         <v>130</v>
       </c>
-      <c r="B134" s="72" t="inlineStr">
-        <is>
-          <t>1784313900119</t>
-        </is>
-      </c>
+      <c r="B134" s="72" t="n"/>
       <c r="C134" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -25806,11 +25326,7 @@
       <c r="A135" s="71" t="n">
         <v>131</v>
       </c>
-      <c r="B135" s="72" t="inlineStr">
-        <is>
-          <t>1784313901096</t>
-        </is>
-      </c>
+      <c r="B135" s="72" t="n"/>
       <c r="C135" t="inlineStr">
         <is>
           <t>wake</t>
@@ -25878,7 +25394,7 @@
       </c>
       <c r="X135" t="inlineStr">
         <is>
-          <t>Disconnected=1</t>
+          <t>Connected=1; Disconnected=1</t>
         </is>
       </c>
     </row>
@@ -25886,11 +25402,7 @@
       <c r="A136" s="71" t="n">
         <v>132</v>
       </c>
-      <c r="B136" s="72" t="inlineStr">
-        <is>
-          <t>1784313900096</t>
-        </is>
-      </c>
+      <c r="B136" s="72" t="n"/>
       <c r="C136" t="inlineStr">
         <is>
           <t>opacity</t>
@@ -25932,7 +25444,7 @@
       </c>
       <c r="L136" t="inlineStr">
         <is>
-          <t>/composition/layers/96/clips/1/video/opacity</t>
+          <t>/composition/layers/96/clips/1/connect</t>
         </is>
       </c>
       <c r="M136" s="71" t="n">
@@ -25962,7 +25474,12 @@
       </c>
       <c r="U136" t="inlineStr">
         <is>
-          <t>/composition/layers/96/clips/1/video/opacity</t>
+          <t>/composition/layers/96/clips/1/connect</t>
+        </is>
+      </c>
+      <c r="X136" t="inlineStr">
+        <is>
+          <t>Connected=1; Disconnected=1</t>
         </is>
       </c>
     </row>
@@ -25970,11 +25487,7 @@
       <c r="A137" s="71" t="n">
         <v>133</v>
       </c>
-      <c r="B137" s="72" t="inlineStr">
-        <is>
-          <t>1784313902096</t>
-        </is>
-      </c>
+      <c r="B137" s="72" t="n"/>
       <c r="C137" t="inlineStr">
         <is>
           <t>motion_y</t>
@@ -26016,7 +25529,7 @@
       </c>
       <c r="L137" t="inlineStr">
         <is>
-          <t>/composition/layers/96/clips/1/video/effects/transform/positiony</t>
+          <t>/composition/layers/96/clips/1/connect</t>
         </is>
       </c>
       <c r="M137" s="71" t="n">
@@ -26046,7 +25559,12 @@
       </c>
       <c r="U137" t="inlineStr">
         <is>
-          <t>/composition/layers/96/clips/1/video/effects/transform/positiony</t>
+          <t>/composition/layers/96/clips/1/connect</t>
+        </is>
+      </c>
+      <c r="X137" t="inlineStr">
+        <is>
+          <t>Connected=1; Disconnected=1</t>
         </is>
       </c>
     </row>
@@ -26054,11 +25572,7 @@
       <c r="A138" s="71" t="n">
         <v>134</v>
       </c>
-      <c r="B138" s="72" t="inlineStr">
-        <is>
-          <t>1784313901112</t>
-        </is>
-      </c>
+      <c r="B138" s="72" t="n"/>
       <c r="C138" t="inlineStr">
         <is>
           <t>wake</t>
@@ -26100,7 +25614,7 @@
       </c>
       <c r="L138" t="inlineStr">
         <is>
-          <t>/composition/layers/112/clips/1/connect</t>
+          <t>/composition/layers/112/clips/1/video/opacity</t>
         </is>
       </c>
       <c r="M138" s="71" t="n">
@@ -26121,7 +25635,7 @@
       </c>
       <c r="U138" t="inlineStr">
         <is>
-          <t>/composition/layers/112/clips/1/connect</t>
+          <t>/composition/layers/112/clips/1/video/opacity</t>
         </is>
       </c>
       <c r="X138" t="inlineStr">
@@ -26134,11 +25648,7 @@
       <c r="A139" s="71" t="n">
         <v>135</v>
       </c>
-      <c r="B139" s="72" t="inlineStr">
-        <is>
-          <t>1784313900112</t>
-        </is>
-      </c>
+      <c r="B139" s="72" t="n"/>
       <c r="C139" t="inlineStr">
         <is>
           <t>opacity</t>
@@ -26218,11 +25728,7 @@
       <c r="A140" s="71" t="n">
         <v>136</v>
       </c>
-      <c r="B140" s="72" t="inlineStr">
-        <is>
-          <t>1784313902112</t>
-        </is>
-      </c>
+      <c r="B140" s="72" t="n"/>
       <c r="C140" t="inlineStr">
         <is>
           <t>motion_rotation</t>
@@ -26264,7 +25770,7 @@
       </c>
       <c r="L140" t="inlineStr">
         <is>
-          <t>/composition/layers/112/clips/1/video/effects/transform/rotationz</t>
+          <t>/composition/layers/112/clips/1/video/opacity</t>
         </is>
       </c>
       <c r="M140" s="71" t="n">
@@ -26294,7 +25800,7 @@
       </c>
       <c r="U140" t="inlineStr">
         <is>
-          <t>/composition/layers/112/clips/1/video/effects/transform/rotationz</t>
+          <t>/composition/layers/112/clips/1/video/opacity</t>
         </is>
       </c>
     </row>
@@ -26302,11 +25808,7 @@
       <c r="A141" s="71" t="n">
         <v>137</v>
       </c>
-      <c r="B141" s="72" t="inlineStr">
-        <is>
-          <t>1784313901095</t>
-        </is>
-      </c>
+      <c r="B141" s="72" t="n"/>
       <c r="C141" t="inlineStr">
         <is>
           <t>wake</t>
@@ -26348,7 +25850,7 @@
       </c>
       <c r="L141" t="inlineStr">
         <is>
-          <t>/composition/layers/95/clips/1/connect</t>
+          <t>/composition/layers/95/clips/1/video/effects/transform/positiony</t>
         </is>
       </c>
       <c r="M141" s="71" t="n">
@@ -26369,7 +25871,7 @@
       </c>
       <c r="U141" t="inlineStr">
         <is>
-          <t>/composition/layers/95/clips/1/connect</t>
+          <t>/composition/layers/95/clips/1/video/effects/transform/positiony</t>
         </is>
       </c>
       <c r="X141" t="inlineStr">
@@ -26382,11 +25884,7 @@
       <c r="A142" s="71" t="n">
         <v>138</v>
       </c>
-      <c r="B142" s="72" t="inlineStr">
-        <is>
-          <t>1784313900095</t>
-        </is>
-      </c>
+      <c r="B142" s="72" t="n"/>
       <c r="C142" t="inlineStr">
         <is>
           <t>opacity</t>
@@ -26428,7 +25926,7 @@
       </c>
       <c r="L142" t="inlineStr">
         <is>
-          <t>/composition/layers/95/clips/1/video/opacity</t>
+          <t>/composition/layers/95/clips/1/video/effects/transform/positiony</t>
         </is>
       </c>
       <c r="M142" s="71" t="n">
@@ -26458,7 +25956,7 @@
       </c>
       <c r="U142" t="inlineStr">
         <is>
-          <t>/composition/layers/95/clips/1/video/opacity</t>
+          <t>/composition/layers/95/clips/1/video/effects/transform/positiony</t>
         </is>
       </c>
     </row>
@@ -26466,11 +25964,7 @@
       <c r="A143" s="71" t="n">
         <v>139</v>
       </c>
-      <c r="B143" s="72" t="inlineStr">
-        <is>
-          <t>1784313902095</t>
-        </is>
-      </c>
+      <c r="B143" s="72" t="n"/>
       <c r="C143" t="inlineStr">
         <is>
           <t>motion_y</t>
@@ -26550,11 +26044,7 @@
       <c r="A144" s="71" t="n">
         <v>140</v>
       </c>
-      <c r="B144" s="72" t="inlineStr">
-        <is>
-          <t>1784313900125</t>
-        </is>
-      </c>
+      <c r="B144" s="72" t="n"/>
       <c r="C144" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -26645,11 +26135,7 @@
       <c r="A145" s="71" t="n">
         <v>141</v>
       </c>
-      <c r="B145" s="72" t="inlineStr">
-        <is>
-          <t>1784313900088</t>
-        </is>
-      </c>
+      <c r="B145" s="72" t="n"/>
       <c r="C145" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -26732,7 +26218,7 @@
       </c>
       <c r="X145" t="inlineStr">
         <is>
-          <t>Connected=0.070866141732283463583; Connected &amp; previewing=0.070866141732283463583; Disconnected=0; Empty=0; Off=0; Previewing=0</t>
+          <t>Connected=1.0; Connected &amp; previewing=1.0; Disconnected=1.0; Empty=0; Off=0; Previewing=0</t>
         </is>
       </c>
     </row>
@@ -26740,11 +26226,7 @@
       <c r="A146" s="71" t="n">
         <v>142</v>
       </c>
-      <c r="B146" s="72" t="inlineStr">
-        <is>
-          <t>1784313900068</t>
-        </is>
-      </c>
+      <c r="B146" s="72" t="n"/>
       <c r="C146" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -26835,11 +26317,7 @@
       <c r="A147" s="71" t="n">
         <v>143</v>
       </c>
-      <c r="B147" s="72" t="inlineStr">
-        <is>
-          <t>1784313900081</t>
-        </is>
-      </c>
+      <c r="B147" s="72" t="n"/>
       <c r="C147" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -26930,11 +26408,7 @@
       <c r="A148" s="71" t="n">
         <v>144</v>
       </c>
-      <c r="B148" s="72" t="inlineStr">
-        <is>
-          <t>1784313900084</t>
-        </is>
-      </c>
+      <c r="B148" s="72" t="n"/>
       <c r="C148" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -27025,11 +26499,7 @@
       <c r="A149" s="71" t="n">
         <v>145</v>
       </c>
-      <c r="B149" s="72" t="inlineStr">
-        <is>
-          <t>1784313900089</t>
-        </is>
-      </c>
+      <c r="B149" s="72" t="n"/>
       <c r="C149" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -27112,7 +26582,7 @@
       </c>
       <c r="X149" t="inlineStr">
         <is>
-          <t>Connected=0.070866141732283463583; Connected &amp; previewing=0.070866141732283463583; Disconnected=0; Empty=0; Off=0; Previewing=0</t>
+          <t>Connected=1.0; Connected &amp; previewing=1.0; Disconnected=1.0; Empty=0; Off=0; Previewing=0</t>
         </is>
       </c>
     </row>
@@ -27120,11 +26590,7 @@
       <c r="A150" s="71" t="n">
         <v>146</v>
       </c>
-      <c r="B150" s="72" t="inlineStr">
-        <is>
-          <t>1784313900074</t>
-        </is>
-      </c>
+      <c r="B150" s="72" t="n"/>
       <c r="C150" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -27215,11 +26681,7 @@
       <c r="A151" s="71" t="n">
         <v>147</v>
       </c>
-      <c r="B151" s="72" t="inlineStr">
-        <is>
-          <t>1784313900076</t>
-        </is>
-      </c>
+      <c r="B151" s="72" t="n"/>
       <c r="C151" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -27310,11 +26772,7 @@
       <c r="A152" s="71" t="n">
         <v>148</v>
       </c>
-      <c r="B152" s="72" t="inlineStr">
-        <is>
-          <t>1784313900127</t>
-        </is>
-      </c>
+      <c r="B152" s="72" t="n"/>
       <c r="C152" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -27405,11 +26863,7 @@
       <c r="A153" s="71" t="n">
         <v>149</v>
       </c>
-      <c r="B153" s="72" t="inlineStr">
-        <is>
-          <t>1784313901116</t>
-        </is>
-      </c>
+      <c r="B153" s="72" t="n"/>
       <c r="C153" t="inlineStr">
         <is>
           <t>wake</t>
@@ -27451,7 +26905,7 @@
       </c>
       <c r="L153" t="inlineStr">
         <is>
-          <t>/composition/layers/116/clips/1/connect</t>
+          <t>/composition/layers/116/clips/1/video/effects/transform/rotationz</t>
         </is>
       </c>
       <c r="M153" s="71" t="n">
@@ -27472,7 +26926,7 @@
       </c>
       <c r="U153" t="inlineStr">
         <is>
-          <t>/composition/layers/116/clips/1/connect</t>
+          <t>/composition/layers/116/clips/1/video/effects/transform/rotationz</t>
         </is>
       </c>
       <c r="X153" t="inlineStr">
@@ -27485,11 +26939,7 @@
       <c r="A154" s="71" t="n">
         <v>150</v>
       </c>
-      <c r="B154" s="72" t="inlineStr">
-        <is>
-          <t>1784313900116</t>
-        </is>
-      </c>
+      <c r="B154" s="72" t="n"/>
       <c r="C154" t="inlineStr">
         <is>
           <t>opacity</t>
@@ -27531,7 +26981,7 @@
       </c>
       <c r="L154" t="inlineStr">
         <is>
-          <t>/composition/layers/116/clips/1/video/opacity</t>
+          <t>/composition/layers/116/clips/1/video/effects/transform/rotationz</t>
         </is>
       </c>
       <c r="M154" s="71" t="n">
@@ -27561,7 +27011,7 @@
       </c>
       <c r="U154" t="inlineStr">
         <is>
-          <t>/composition/layers/116/clips/1/video/opacity</t>
+          <t>/composition/layers/116/clips/1/video/effects/transform/rotationz</t>
         </is>
       </c>
     </row>
@@ -27569,11 +27019,7 @@
       <c r="A155" s="71" t="n">
         <v>151</v>
       </c>
-      <c r="B155" s="72" t="inlineStr">
-        <is>
-          <t>1784313902116</t>
-        </is>
-      </c>
+      <c r="B155" s="72" t="n"/>
       <c r="C155" t="inlineStr">
         <is>
           <t>motion_rotation</t>
@@ -27653,11 +27099,7 @@
       <c r="A156" s="71" t="n">
         <v>152</v>
       </c>
-      <c r="B156" s="72" t="inlineStr">
-        <is>
-          <t>1784313900124</t>
-        </is>
-      </c>
+      <c r="B156" s="72" t="n"/>
       <c r="C156" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -27748,11 +27190,7 @@
       <c r="A157" s="71" t="n">
         <v>153</v>
       </c>
-      <c r="B157" s="72" t="inlineStr">
-        <is>
-          <t>1784313901115</t>
-        </is>
-      </c>
+      <c r="B157" s="72" t="n"/>
       <c r="C157" t="inlineStr">
         <is>
           <t>wake</t>
@@ -27820,7 +27258,7 @@
       </c>
       <c r="X157" t="inlineStr">
         <is>
-          <t>Disconnected=1</t>
+          <t>Connected=1; Disconnected=1</t>
         </is>
       </c>
     </row>
@@ -27828,11 +27266,7 @@
       <c r="A158" s="71" t="n">
         <v>154</v>
       </c>
-      <c r="B158" s="72" t="inlineStr">
-        <is>
-          <t>1784313900115</t>
-        </is>
-      </c>
+      <c r="B158" s="72" t="n"/>
       <c r="C158" t="inlineStr">
         <is>
           <t>opacity</t>
@@ -27874,7 +27308,7 @@
       </c>
       <c r="L158" t="inlineStr">
         <is>
-          <t>/composition/layers/115/clips/1/video/opacity</t>
+          <t>/composition/layers/115/clips/1/connect</t>
         </is>
       </c>
       <c r="M158" s="71" t="n">
@@ -27904,7 +27338,12 @@
       </c>
       <c r="U158" t="inlineStr">
         <is>
-          <t>/composition/layers/115/clips/1/video/opacity</t>
+          <t>/composition/layers/115/clips/1/connect</t>
+        </is>
+      </c>
+      <c r="X158" t="inlineStr">
+        <is>
+          <t>Connected=1; Disconnected=1</t>
         </is>
       </c>
     </row>
@@ -27912,11 +27351,7 @@
       <c r="A159" s="71" t="n">
         <v>155</v>
       </c>
-      <c r="B159" s="72" t="inlineStr">
-        <is>
-          <t>1784313902115</t>
-        </is>
-      </c>
+      <c r="B159" s="72" t="n"/>
       <c r="C159" t="inlineStr">
         <is>
           <t>motion_rotation</t>
@@ -27958,7 +27393,7 @@
       </c>
       <c r="L159" t="inlineStr">
         <is>
-          <t>/composition/layers/115/clips/1/video/effects/transform/rotationz</t>
+          <t>/composition/layers/115/clips/1/connect</t>
         </is>
       </c>
       <c r="M159" s="71" t="n">
@@ -27988,7 +27423,12 @@
       </c>
       <c r="U159" t="inlineStr">
         <is>
-          <t>/composition/layers/115/clips/1/video/effects/transform/rotationz</t>
+          <t>/composition/layers/115/clips/1/connect</t>
+        </is>
+      </c>
+      <c r="X159" t="inlineStr">
+        <is>
+          <t>Connected=1; Disconnected=1</t>
         </is>
       </c>
     </row>
@@ -27996,11 +27436,7 @@
       <c r="A160" s="71" t="n">
         <v>156</v>
       </c>
-      <c r="B160" s="72" t="inlineStr">
-        <is>
-          <t>1784313900093</t>
-        </is>
-      </c>
+      <c r="B160" s="72" t="n"/>
       <c r="C160" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -28083,7 +27519,7 @@
       </c>
       <c r="X160" t="inlineStr">
         <is>
-          <t>Connected=0.070866141732283463583; Connected &amp; previewing=0.070866141732283463583; Disconnected=0; Empty=0; Off=0; Previewing=0</t>
+          <t>Connected=1.0; Connected &amp; previewing=1.0; Disconnected=1.0; Empty=0; Off=0; Previewing=0</t>
         </is>
       </c>
     </row>
@@ -28091,11 +27527,7 @@
       <c r="A161" s="71" t="n">
         <v>157</v>
       </c>
-      <c r="B161" s="72" t="inlineStr">
-        <is>
-          <t>1784313901097</t>
-        </is>
-      </c>
+      <c r="B161" s="72" t="n"/>
       <c r="C161" t="inlineStr">
         <is>
           <t>wake</t>
@@ -28163,7 +27595,7 @@
       </c>
       <c r="X161" t="inlineStr">
         <is>
-          <t>Disconnected=1</t>
+          <t>Connected=1; Disconnected=1</t>
         </is>
       </c>
     </row>
@@ -28171,11 +27603,7 @@
       <c r="A162" s="71" t="n">
         <v>158</v>
       </c>
-      <c r="B162" s="72" t="inlineStr">
-        <is>
-          <t>1784313900097</t>
-        </is>
-      </c>
+      <c r="B162" s="72" t="n"/>
       <c r="C162" t="inlineStr">
         <is>
           <t>opacity</t>
@@ -28217,7 +27645,7 @@
       </c>
       <c r="L162" t="inlineStr">
         <is>
-          <t>/composition/layers/97/clips/1/video/opacity</t>
+          <t>/composition/layers/97/clips/1/connect</t>
         </is>
       </c>
       <c r="M162" s="71" t="n">
@@ -28247,7 +27675,12 @@
       </c>
       <c r="U162" t="inlineStr">
         <is>
-          <t>/composition/layers/97/clips/1/video/opacity</t>
+          <t>/composition/layers/97/clips/1/connect</t>
+        </is>
+      </c>
+      <c r="X162" t="inlineStr">
+        <is>
+          <t>Connected=1; Disconnected=1</t>
         </is>
       </c>
     </row>
@@ -28255,11 +27688,7 @@
       <c r="A163" s="71" t="n">
         <v>159</v>
       </c>
-      <c r="B163" s="72" t="inlineStr">
-        <is>
-          <t>1784313902097</t>
-        </is>
-      </c>
+      <c r="B163" s="72" t="n"/>
       <c r="C163" t="inlineStr">
         <is>
           <t>motion_y</t>
@@ -28301,7 +27730,7 @@
       </c>
       <c r="L163" t="inlineStr">
         <is>
-          <t>/composition/layers/97/clips/1/video/effects/transform/positiony</t>
+          <t>/composition/layers/97/clips/1/connect</t>
         </is>
       </c>
       <c r="M163" s="71" t="n">
@@ -28331,7 +27760,12 @@
       </c>
       <c r="U163" t="inlineStr">
         <is>
-          <t>/composition/layers/97/clips/1/video/effects/transform/positiony</t>
+          <t>/composition/layers/97/clips/1/connect</t>
+        </is>
+      </c>
+      <c r="X163" t="inlineStr">
+        <is>
+          <t>Connected=1; Disconnected=1</t>
         </is>
       </c>
     </row>
@@ -28339,11 +27773,7 @@
       <c r="A164" s="71" t="n">
         <v>160</v>
       </c>
-      <c r="B164" s="72" t="inlineStr">
-        <is>
-          <t>1784313901102</t>
-        </is>
-      </c>
+      <c r="B164" s="72" t="n"/>
       <c r="C164" t="inlineStr">
         <is>
           <t>wake</t>
@@ -28385,7 +27815,7 @@
       </c>
       <c r="L164" t="inlineStr">
         <is>
-          <t>/composition/layers/102/clips/1/connect</t>
+          <t>/composition/layers/102/clips/1/video/effects/transform/rotationz</t>
         </is>
       </c>
       <c r="M164" s="71" t="n">
@@ -28406,7 +27836,7 @@
       </c>
       <c r="U164" t="inlineStr">
         <is>
-          <t>/composition/layers/102/clips/1/connect</t>
+          <t>/composition/layers/102/clips/1/video/effects/transform/rotationz</t>
         </is>
       </c>
       <c r="X164" t="inlineStr">
@@ -28419,11 +27849,7 @@
       <c r="A165" s="71" t="n">
         <v>161</v>
       </c>
-      <c r="B165" s="72" t="inlineStr">
-        <is>
-          <t>1784313900102</t>
-        </is>
-      </c>
+      <c r="B165" s="72" t="n"/>
       <c r="C165" t="inlineStr">
         <is>
           <t>opacity</t>
@@ -28465,7 +27891,7 @@
       </c>
       <c r="L165" t="inlineStr">
         <is>
-          <t>/composition/layers/102/clips/1/video/opacity</t>
+          <t>/composition/layers/102/clips/1/video/effects/transform/rotationz</t>
         </is>
       </c>
       <c r="M165" s="71" t="n">
@@ -28495,7 +27921,7 @@
       </c>
       <c r="U165" t="inlineStr">
         <is>
-          <t>/composition/layers/102/clips/1/video/opacity</t>
+          <t>/composition/layers/102/clips/1/video/effects/transform/rotationz</t>
         </is>
       </c>
     </row>
@@ -28503,11 +27929,7 @@
       <c r="A166" s="71" t="n">
         <v>162</v>
       </c>
-      <c r="B166" s="72" t="inlineStr">
-        <is>
-          <t>1784313902102</t>
-        </is>
-      </c>
+      <c r="B166" s="72" t="n"/>
       <c r="C166" t="inlineStr">
         <is>
           <t>motion_rotation</t>
@@ -28587,11 +28009,7 @@
       <c r="A167" s="71" t="n">
         <v>163</v>
       </c>
-      <c r="B167" s="72" t="inlineStr">
-        <is>
-          <t>1784313901101</t>
-        </is>
-      </c>
+      <c r="B167" s="72" t="n"/>
       <c r="C167" t="inlineStr">
         <is>
           <t>wake</t>
@@ -28659,7 +28077,7 @@
       </c>
       <c r="X167" t="inlineStr">
         <is>
-          <t>Disconnected=1</t>
+          <t>Connected=1; Disconnected=1</t>
         </is>
       </c>
     </row>
@@ -28667,11 +28085,7 @@
       <c r="A168" s="71" t="n">
         <v>164</v>
       </c>
-      <c r="B168" s="72" t="inlineStr">
-        <is>
-          <t>1784313900101</t>
-        </is>
-      </c>
+      <c r="B168" s="72" t="n"/>
       <c r="C168" t="inlineStr">
         <is>
           <t>opacity</t>
@@ -28713,7 +28127,7 @@
       </c>
       <c r="L168" t="inlineStr">
         <is>
-          <t>/composition/layers/101/clips/1/video/opacity</t>
+          <t>/composition/layers/101/clips/1/connect</t>
         </is>
       </c>
       <c r="M168" s="71" t="n">
@@ -28743,7 +28157,12 @@
       </c>
       <c r="U168" t="inlineStr">
         <is>
-          <t>/composition/layers/101/clips/1/video/opacity</t>
+          <t>/composition/layers/101/clips/1/connect</t>
+        </is>
+      </c>
+      <c r="X168" t="inlineStr">
+        <is>
+          <t>Connected=1; Disconnected=1</t>
         </is>
       </c>
     </row>
@@ -28751,11 +28170,7 @@
       <c r="A169" s="71" t="n">
         <v>165</v>
       </c>
-      <c r="B169" s="72" t="inlineStr">
-        <is>
-          <t>1784313902101</t>
-        </is>
-      </c>
+      <c r="B169" s="72" t="n"/>
       <c r="C169" t="inlineStr">
         <is>
           <t>motion_y</t>
@@ -28797,7 +28212,7 @@
       </c>
       <c r="L169" t="inlineStr">
         <is>
-          <t>/composition/layers/101/clips/1/video/effects/transform/positiony</t>
+          <t>/composition/layers/101/clips/1/connect</t>
         </is>
       </c>
       <c r="M169" s="71" t="n">
@@ -28827,7 +28242,12 @@
       </c>
       <c r="U169" t="inlineStr">
         <is>
-          <t>/composition/layers/101/clips/1/video/effects/transform/positiony</t>
+          <t>/composition/layers/101/clips/1/connect</t>
+        </is>
+      </c>
+      <c r="X169" t="inlineStr">
+        <is>
+          <t>Connected=1; Disconnected=1</t>
         </is>
       </c>
     </row>
@@ -28835,11 +28255,7 @@
       <c r="A170" s="71" t="n">
         <v>166</v>
       </c>
-      <c r="B170" s="72" t="inlineStr">
-        <is>
-          <t>1784313901098</t>
-        </is>
-      </c>
+      <c r="B170" s="72" t="n"/>
       <c r="C170" t="inlineStr">
         <is>
           <t>wake</t>
@@ -28907,7 +28323,7 @@
       </c>
       <c r="X170" t="inlineStr">
         <is>
-          <t>Disconnected=1</t>
+          <t>Connected=1; Disconnected=1</t>
         </is>
       </c>
     </row>
@@ -28915,11 +28331,7 @@
       <c r="A171" s="71" t="n">
         <v>167</v>
       </c>
-      <c r="B171" s="72" t="inlineStr">
-        <is>
-          <t>1784313900098</t>
-        </is>
-      </c>
+      <c r="B171" s="72" t="n"/>
       <c r="C171" t="inlineStr">
         <is>
           <t>opacity</t>
@@ -28961,7 +28373,7 @@
       </c>
       <c r="L171" t="inlineStr">
         <is>
-          <t>/composition/layers/98/clips/1/video/opacity</t>
+          <t>/composition/layers/98/clips/1/connect</t>
         </is>
       </c>
       <c r="M171" s="71" t="n">
@@ -28991,7 +28403,12 @@
       </c>
       <c r="U171" t="inlineStr">
         <is>
-          <t>/composition/layers/98/clips/1/video/opacity</t>
+          <t>/composition/layers/98/clips/1/connect</t>
+        </is>
+      </c>
+      <c r="X171" t="inlineStr">
+        <is>
+          <t>Connected=1; Disconnected=1</t>
         </is>
       </c>
     </row>
@@ -28999,11 +28416,7 @@
       <c r="A172" s="71" t="n">
         <v>168</v>
       </c>
-      <c r="B172" s="72" t="inlineStr">
-        <is>
-          <t>1784313902098</t>
-        </is>
-      </c>
+      <c r="B172" s="72" t="n"/>
       <c r="C172" t="inlineStr">
         <is>
           <t>motion_y</t>
@@ -29045,7 +28458,7 @@
       </c>
       <c r="L172" t="inlineStr">
         <is>
-          <t>/composition/layers/98/clips/1/video/effects/transform/positiony</t>
+          <t>/composition/layers/98/clips/1/connect</t>
         </is>
       </c>
       <c r="M172" s="71" t="n">
@@ -29075,7 +28488,12 @@
       </c>
       <c r="U172" t="inlineStr">
         <is>
-          <t>/composition/layers/98/clips/1/video/effects/transform/positiony</t>
+          <t>/composition/layers/98/clips/1/connect</t>
+        </is>
+      </c>
+      <c r="X172" t="inlineStr">
+        <is>
+          <t>Connected=1; Disconnected=1</t>
         </is>
       </c>
     </row>
@@ -29083,11 +28501,7 @@
       <c r="A173" s="71" t="n">
         <v>169</v>
       </c>
-      <c r="B173" s="72" t="inlineStr">
-        <is>
-          <t>1784313901107</t>
-        </is>
-      </c>
+      <c r="B173" s="72" t="n"/>
       <c r="C173" t="inlineStr">
         <is>
           <t>wake</t>
@@ -29129,7 +28543,7 @@
       </c>
       <c r="L173" t="inlineStr">
         <is>
-          <t>/composition/layers/107/clips/1/connect</t>
+          <t>/composition/layers/107/clips/1/video/opacity</t>
         </is>
       </c>
       <c r="M173" s="71" t="n">
@@ -29150,7 +28564,7 @@
       </c>
       <c r="U173" t="inlineStr">
         <is>
-          <t>/composition/layers/107/clips/1/connect</t>
+          <t>/composition/layers/107/clips/1/video/opacity</t>
         </is>
       </c>
       <c r="X173" t="inlineStr">
@@ -29163,11 +28577,7 @@
       <c r="A174" s="71" t="n">
         <v>170</v>
       </c>
-      <c r="B174" s="72" t="inlineStr">
-        <is>
-          <t>1784313900107</t>
-        </is>
-      </c>
+      <c r="B174" s="72" t="n"/>
       <c r="C174" t="inlineStr">
         <is>
           <t>opacity</t>
@@ -29247,11 +28657,7 @@
       <c r="A175" s="71" t="n">
         <v>171</v>
       </c>
-      <c r="B175" s="72" t="inlineStr">
-        <is>
-          <t>1784313902107</t>
-        </is>
-      </c>
+      <c r="B175" s="72" t="n"/>
       <c r="C175" t="inlineStr">
         <is>
           <t>motion_rotation</t>
@@ -29293,7 +28699,7 @@
       </c>
       <c r="L175" t="inlineStr">
         <is>
-          <t>/composition/layers/107/clips/1/video/effects/transform/rotationz</t>
+          <t>/composition/layers/107/clips/1/video/opacity</t>
         </is>
       </c>
       <c r="M175" s="71" t="n">
@@ -29323,7 +28729,7 @@
       </c>
       <c r="U175" t="inlineStr">
         <is>
-          <t>/composition/layers/107/clips/1/video/effects/transform/rotationz</t>
+          <t>/composition/layers/107/clips/1/video/opacity</t>
         </is>
       </c>
     </row>
@@ -29331,11 +28737,7 @@
       <c r="A176" s="71" t="n">
         <v>172</v>
       </c>
-      <c r="B176" s="72" t="inlineStr">
-        <is>
-          <t>1784313900130</t>
-        </is>
-      </c>
+      <c r="B176" s="72" t="n"/>
       <c r="C176" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -29426,11 +28828,7 @@
       <c r="A177" s="71" t="n">
         <v>173</v>
       </c>
-      <c r="B177" s="72" t="inlineStr">
-        <is>
-          <t>1784313900121</t>
-        </is>
-      </c>
+      <c r="B177" s="72" t="n"/>
       <c r="C177" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -29521,11 +28919,7 @@
       <c r="A178" s="71" t="n">
         <v>174</v>
       </c>
-      <c r="B178" s="72" t="inlineStr">
-        <is>
-          <t>1784313901111</t>
-        </is>
-      </c>
+      <c r="B178" s="72" t="n"/>
       <c r="C178" t="inlineStr">
         <is>
           <t>wake</t>
@@ -29567,7 +28961,7 @@
       </c>
       <c r="L178" t="inlineStr">
         <is>
-          <t>/composition/layers/111/clips/1/connect</t>
+          <t>/composition/layers/111/clips/1/video/effects/transform/rotationz</t>
         </is>
       </c>
       <c r="M178" s="71" t="n">
@@ -29588,7 +28982,7 @@
       </c>
       <c r="U178" t="inlineStr">
         <is>
-          <t>/composition/layers/111/clips/1/connect</t>
+          <t>/composition/layers/111/clips/1/video/effects/transform/rotationz</t>
         </is>
       </c>
       <c r="X178" t="inlineStr">
@@ -29601,11 +28995,7 @@
       <c r="A179" s="71" t="n">
         <v>175</v>
       </c>
-      <c r="B179" s="72" t="inlineStr">
-        <is>
-          <t>1784313900111</t>
-        </is>
-      </c>
+      <c r="B179" s="72" t="n"/>
       <c r="C179" t="inlineStr">
         <is>
           <t>opacity</t>
@@ -29647,7 +29037,7 @@
       </c>
       <c r="L179" t="inlineStr">
         <is>
-          <t>/composition/layers/111/clips/1/video/opacity</t>
+          <t>/composition/layers/111/clips/1/video/effects/transform/rotationz</t>
         </is>
       </c>
       <c r="M179" s="71" t="n">
@@ -29677,7 +29067,7 @@
       </c>
       <c r="U179" t="inlineStr">
         <is>
-          <t>/composition/layers/111/clips/1/video/opacity</t>
+          <t>/composition/layers/111/clips/1/video/effects/transform/rotationz</t>
         </is>
       </c>
     </row>
@@ -29685,11 +29075,7 @@
       <c r="A180" s="71" t="n">
         <v>176</v>
       </c>
-      <c r="B180" s="72" t="inlineStr">
-        <is>
-          <t>1784313902111</t>
-        </is>
-      </c>
+      <c r="B180" s="72" t="n"/>
       <c r="C180" t="inlineStr">
         <is>
           <t>motion_rotation</t>
@@ -29769,11 +29155,7 @@
       <c r="A181" s="71" t="n">
         <v>177</v>
       </c>
-      <c r="B181" s="72" t="inlineStr">
-        <is>
-          <t>1784313900128</t>
-        </is>
-      </c>
+      <c r="B181" s="72" t="n"/>
       <c r="C181" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -29864,11 +29246,7 @@
       <c r="A182" s="71" t="n">
         <v>178</v>
       </c>
-      <c r="B182" s="72" t="inlineStr">
-        <is>
-          <t>1784313901110</t>
-        </is>
-      </c>
+      <c r="B182" s="72" t="n"/>
       <c r="C182" t="inlineStr">
         <is>
           <t>wake</t>
@@ -29936,7 +29314,7 @@
       </c>
       <c r="X182" t="inlineStr">
         <is>
-          <t>Disconnected=1</t>
+          <t>Connected=1; Disconnected=1</t>
         </is>
       </c>
     </row>
@@ -29944,11 +29322,7 @@
       <c r="A183" s="71" t="n">
         <v>179</v>
       </c>
-      <c r="B183" s="72" t="inlineStr">
-        <is>
-          <t>1784313900110</t>
-        </is>
-      </c>
+      <c r="B183" s="72" t="n"/>
       <c r="C183" t="inlineStr">
         <is>
           <t>opacity</t>
@@ -29990,7 +29364,7 @@
       </c>
       <c r="L183" t="inlineStr">
         <is>
-          <t>/composition/layers/110/clips/1/video/opacity</t>
+          <t>/composition/layers/110/clips/1/connect</t>
         </is>
       </c>
       <c r="M183" s="71" t="n">
@@ -30020,7 +29394,12 @@
       </c>
       <c r="U183" t="inlineStr">
         <is>
-          <t>/composition/layers/110/clips/1/video/opacity</t>
+          <t>/composition/layers/110/clips/1/connect</t>
+        </is>
+      </c>
+      <c r="X183" t="inlineStr">
+        <is>
+          <t>Connected=1; Disconnected=1</t>
         </is>
       </c>
     </row>
@@ -30028,11 +29407,7 @@
       <c r="A184" s="71" t="n">
         <v>180</v>
       </c>
-      <c r="B184" s="72" t="inlineStr">
-        <is>
-          <t>1784313902110</t>
-        </is>
-      </c>
+      <c r="B184" s="72" t="n"/>
       <c r="C184" t="inlineStr">
         <is>
           <t>motion_rotation</t>
@@ -30074,7 +29449,7 @@
       </c>
       <c r="L184" t="inlineStr">
         <is>
-          <t>/composition/layers/110/clips/1/video/effects/transform/rotationz</t>
+          <t>/composition/layers/110/clips/1/connect</t>
         </is>
       </c>
       <c r="M184" s="71" t="n">
@@ -30104,7 +29479,12 @@
       </c>
       <c r="U184" t="inlineStr">
         <is>
-          <t>/composition/layers/110/clips/1/video/effects/transform/rotationz</t>
+          <t>/composition/layers/110/clips/1/connect</t>
+        </is>
+      </c>
+      <c r="X184" t="inlineStr">
+        <is>
+          <t>Connected=1; Disconnected=1</t>
         </is>
       </c>
     </row>
@@ -30112,11 +29492,7 @@
       <c r="A185" s="71" t="n">
         <v>181</v>
       </c>
-      <c r="B185" s="72" t="inlineStr">
-        <is>
-          <t>1784313900131</t>
-        </is>
-      </c>
+      <c r="B185" s="72" t="n"/>
       <c r="C185" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -30207,11 +29583,7 @@
       <c r="A186" s="71" t="n">
         <v>182</v>
       </c>
-      <c r="B186" s="72" t="inlineStr">
-        <is>
-          <t>1784313901105</t>
-        </is>
-      </c>
+      <c r="B186" s="72" t="n"/>
       <c r="C186" t="inlineStr">
         <is>
           <t>wake</t>
@@ -30253,7 +29625,7 @@
       </c>
       <c r="L186" t="inlineStr">
         <is>
-          <t>/composition/layers/105/clips/1/connect</t>
+          <t>/composition/layers/105/clips/1/video/opacity</t>
         </is>
       </c>
       <c r="M186" s="71" t="n">
@@ -30274,7 +29646,7 @@
       </c>
       <c r="U186" t="inlineStr">
         <is>
-          <t>/composition/layers/105/clips/1/connect</t>
+          <t>/composition/layers/105/clips/1/video/opacity</t>
         </is>
       </c>
       <c r="X186" t="inlineStr">
@@ -30287,11 +29659,7 @@
       <c r="A187" s="71" t="n">
         <v>183</v>
       </c>
-      <c r="B187" s="72" t="inlineStr">
-        <is>
-          <t>1784313900105</t>
-        </is>
-      </c>
+      <c r="B187" s="72" t="n"/>
       <c r="C187" t="inlineStr">
         <is>
           <t>opacity</t>
@@ -30371,11 +29739,7 @@
       <c r="A188" s="71" t="n">
         <v>184</v>
       </c>
-      <c r="B188" s="72" t="inlineStr">
-        <is>
-          <t>1784313902105</t>
-        </is>
-      </c>
+      <c r="B188" s="72" t="n"/>
       <c r="C188" t="inlineStr">
         <is>
           <t>motion_rotation</t>
@@ -30417,7 +29781,7 @@
       </c>
       <c r="L188" t="inlineStr">
         <is>
-          <t>/composition/layers/105/clips/1/video/effects/transform/rotationz</t>
+          <t>/composition/layers/105/clips/1/video/opacity</t>
         </is>
       </c>
       <c r="M188" s="71" t="n">
@@ -30447,7 +29811,7 @@
       </c>
       <c r="U188" t="inlineStr">
         <is>
-          <t>/composition/layers/105/clips/1/video/effects/transform/rotationz</t>
+          <t>/composition/layers/105/clips/1/video/opacity</t>
         </is>
       </c>
     </row>
@@ -30455,11 +29819,7 @@
       <c r="A189" s="71" t="n">
         <v>185</v>
       </c>
-      <c r="B189" s="72" t="inlineStr">
-        <is>
-          <t>1784313901117</t>
-        </is>
-      </c>
+      <c r="B189" s="72" t="n"/>
       <c r="C189" t="inlineStr">
         <is>
           <t>wake</t>
@@ -30527,7 +29887,7 @@
       </c>
       <c r="X189" t="inlineStr">
         <is>
-          <t>Disconnected=1</t>
+          <t>Connected=1; Disconnected=1</t>
         </is>
       </c>
     </row>
@@ -30535,11 +29895,7 @@
       <c r="A190" s="71" t="n">
         <v>186</v>
       </c>
-      <c r="B190" s="72" t="inlineStr">
-        <is>
-          <t>1784313900117</t>
-        </is>
-      </c>
+      <c r="B190" s="72" t="n"/>
       <c r="C190" t="inlineStr">
         <is>
           <t>opacity</t>
@@ -30581,7 +29937,7 @@
       </c>
       <c r="L190" t="inlineStr">
         <is>
-          <t>/composition/layers/117/clips/1/video/opacity</t>
+          <t>/composition/layers/117/clips/1/connect</t>
         </is>
       </c>
       <c r="M190" s="71" t="n">
@@ -30611,7 +29967,12 @@
       </c>
       <c r="U190" t="inlineStr">
         <is>
-          <t>/composition/layers/117/clips/1/video/opacity</t>
+          <t>/composition/layers/117/clips/1/connect</t>
+        </is>
+      </c>
+      <c r="X190" t="inlineStr">
+        <is>
+          <t>Connected=1; Disconnected=1</t>
         </is>
       </c>
     </row>
@@ -30619,11 +29980,7 @@
       <c r="A191" s="71" t="n">
         <v>187</v>
       </c>
-      <c r="B191" s="72" t="inlineStr">
-        <is>
-          <t>1784313902117</t>
-        </is>
-      </c>
+      <c r="B191" s="72" t="n"/>
       <c r="C191" t="inlineStr">
         <is>
           <t>motion_rotation</t>
@@ -30665,7 +30022,7 @@
       </c>
       <c r="L191" t="inlineStr">
         <is>
-          <t>/composition/layers/117/clips/1/video/effects/transform/rotationz</t>
+          <t>/composition/layers/117/clips/1/connect</t>
         </is>
       </c>
       <c r="M191" s="71" t="n">
@@ -30695,7 +30052,12 @@
       </c>
       <c r="U191" t="inlineStr">
         <is>
-          <t>/composition/layers/117/clips/1/video/effects/transform/rotationz</t>
+          <t>/composition/layers/117/clips/1/connect</t>
+        </is>
+      </c>
+      <c r="X191" t="inlineStr">
+        <is>
+          <t>Connected=1; Disconnected=1</t>
         </is>
       </c>
     </row>
@@ -30703,11 +30065,7 @@
       <c r="A192" s="71" t="n">
         <v>188</v>
       </c>
-      <c r="B192" s="72" t="inlineStr">
-        <is>
-          <t>1784313900132</t>
-        </is>
-      </c>
+      <c r="B192" s="72" t="n"/>
       <c r="C192" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -30798,11 +30156,7 @@
       <c r="A193" s="71" t="n">
         <v>189</v>
       </c>
-      <c r="B193" s="72" t="inlineStr">
-        <is>
-          <t>1784313900134</t>
-        </is>
-      </c>
+      <c r="B193" s="72" t="n"/>
       <c r="C193" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -30893,11 +30247,7 @@
       <c r="A194" s="71" t="n">
         <v>190</v>
       </c>
-      <c r="B194" s="72" t="inlineStr">
-        <is>
-          <t>1784313900118</t>
-        </is>
-      </c>
+      <c r="B194" s="72" t="n"/>
       <c r="C194" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -30988,11 +30338,7 @@
       <c r="A195" s="71" t="n">
         <v>191</v>
       </c>
-      <c r="B195" s="72" t="inlineStr">
-        <is>
-          <t>1784313900133</t>
-        </is>
-      </c>
+      <c r="B195" s="72" t="n"/>
       <c r="C195" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -31083,11 +30429,7 @@
       <c r="A196" s="71" t="n">
         <v>192</v>
       </c>
-      <c r="B196" s="72" t="inlineStr">
-        <is>
-          <t>1784313900129</t>
-        </is>
-      </c>
+      <c r="B196" s="72" t="n"/>
       <c r="C196" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -31178,11 +30520,7 @@
       <c r="A197" s="71" t="n">
         <v>193</v>
       </c>
-      <c r="B197" s="72" t="inlineStr">
-        <is>
-          <t>1784313901103</t>
-        </is>
-      </c>
+      <c r="B197" s="72" t="n"/>
       <c r="C197" t="inlineStr">
         <is>
           <t>wake</t>
@@ -31224,7 +30562,7 @@
       </c>
       <c r="L197" t="inlineStr">
         <is>
-          <t>/composition/layers/103/clips/1/connect</t>
+          <t>/composition/layers/103/clips/1/video/effects/transform/rotationz</t>
         </is>
       </c>
       <c r="M197" s="71" t="n">
@@ -31245,7 +30583,7 @@
       </c>
       <c r="U197" t="inlineStr">
         <is>
-          <t>/composition/layers/103/clips/1/connect</t>
+          <t>/composition/layers/103/clips/1/video/effects/transform/rotationz</t>
         </is>
       </c>
       <c r="X197" t="inlineStr">
@@ -31258,11 +30596,7 @@
       <c r="A198" s="71" t="n">
         <v>194</v>
       </c>
-      <c r="B198" s="72" t="inlineStr">
-        <is>
-          <t>1784313900103</t>
-        </is>
-      </c>
+      <c r="B198" s="72" t="n"/>
       <c r="C198" t="inlineStr">
         <is>
           <t>opacity</t>
@@ -31304,7 +30638,7 @@
       </c>
       <c r="L198" t="inlineStr">
         <is>
-          <t>/composition/layers/103/clips/1/video/opacity</t>
+          <t>/composition/layers/103/clips/1/video/effects/transform/rotationz</t>
         </is>
       </c>
       <c r="M198" s="71" t="n">
@@ -31334,7 +30668,7 @@
       </c>
       <c r="U198" t="inlineStr">
         <is>
-          <t>/composition/layers/103/clips/1/video/opacity</t>
+          <t>/composition/layers/103/clips/1/video/effects/transform/rotationz</t>
         </is>
       </c>
     </row>
@@ -31342,11 +30676,7 @@
       <c r="A199" s="71" t="n">
         <v>195</v>
       </c>
-      <c r="B199" s="72" t="inlineStr">
-        <is>
-          <t>1784313902103</t>
-        </is>
-      </c>
+      <c r="B199" s="72" t="n"/>
       <c r="C199" t="inlineStr">
         <is>
           <t>motion_rotation</t>
@@ -31426,11 +30756,7 @@
       <c r="A200" s="71" t="n">
         <v>196</v>
       </c>
-      <c r="B200" s="72" t="inlineStr">
-        <is>
-          <t>1784313900126</t>
-        </is>
-      </c>
+      <c r="B200" s="72" t="n"/>
       <c r="C200" t="inlineStr">
         <is>
           <t>button_connect</t>
@@ -31521,11 +30847,7 @@
       <c r="A201" s="71" t="n">
         <v>197</v>
       </c>
-      <c r="B201" s="72" t="inlineStr">
-        <is>
-          <t>1784313901108</t>
-        </is>
-      </c>
+      <c r="B201" s="72" t="n"/>
       <c r="C201" t="inlineStr">
         <is>
           <t>wake</t>
@@ -31567,7 +30889,7 @@
       </c>
       <c r="L201" t="inlineStr">
         <is>
-          <t>/composition/layers/108/clips/1/connect</t>
+          <t>/composition/layers/108/clips/1/video/effects/transform/rotationz</t>
         </is>
       </c>
       <c r="M201" s="71" t="n">
@@ -31588,7 +30910,7 @@
       </c>
       <c r="U201" t="inlineStr">
         <is>
-          <t>/composition/layers/108/clips/1/connect</t>
+          <t>/composition/layers/108/clips/1/video/effects/transform/rotationz</t>
         </is>
       </c>
       <c r="X201" t="inlineStr">
@@ -31601,11 +30923,7 @@
       <c r="A202" s="71" t="n">
         <v>198</v>
       </c>
-      <c r="B202" s="72" t="inlineStr">
-        <is>
-          <t>1784313900108</t>
-        </is>
-      </c>
+      <c r="B202" s="72" t="n"/>
       <c r="C202" t="inlineStr">
         <is>
           <t>opacity</t>
@@ -31647,7 +30965,7 @@
       </c>
       <c r="L202" t="inlineStr">
         <is>
-          <t>/composition/layers/108/clips/1/video/opacity</t>
+          <t>/composition/layers/108/clips/1/video/effects/transform/rotationz</t>
         </is>
       </c>
       <c r="M202" s="71" t="n">
@@ -31677,7 +30995,7 @@
       </c>
       <c r="U202" t="inlineStr">
         <is>
-          <t>/composition/layers/108/clips/1/video/opacity</t>
+          <t>/composition/layers/108/clips/1/video/effects/transform/rotationz</t>
         </is>
       </c>
     </row>
@@ -31685,11 +31003,7 @@
       <c r="A203" s="71" t="n">
         <v>199</v>
       </c>
-      <c r="B203" s="72" t="inlineStr">
-        <is>
-          <t>1784313902108</t>
-        </is>
-      </c>
+      <c r="B203" s="72" t="n"/>
       <c r="C203" t="inlineStr">
         <is>
           <t>motion_rotation</t>
@@ -31769,11 +31083,7 @@
       <c r="A204" s="71" t="n">
         <v>200</v>
       </c>
-      <c r="B204" s="72" t="inlineStr">
-        <is>
-          <t>1784313901100</t>
-        </is>
-      </c>
+      <c r="B204" s="72" t="n"/>
       <c r="C204" t="inlineStr">
         <is>
           <t>wake</t>
@@ -31841,7 +31151,7 @@
       </c>
       <c r="X204" t="inlineStr">
         <is>
-          <t>Disconnected=1</t>
+          <t>Connected=1; Disconnected=1</t>
         </is>
       </c>
     </row>
@@ -31849,11 +31159,7 @@
       <c r="A205" s="71" t="n">
         <v>201</v>
       </c>
-      <c r="B205" s="72" t="inlineStr">
-        <is>
-          <t>1784313900100</t>
-        </is>
-      </c>
+      <c r="B205" s="72" t="n"/>
       <c r="C205" t="inlineStr">
         <is>
           <t>opacity</t>
@@ -31895,7 +31201,7 @@
       </c>
       <c r="L205" t="inlineStr">
         <is>
-          <t>/composition/layers/100/clips/1/video/opacity</t>
+          <t>/composition/layers/100/clips/1/connect</t>
         </is>
       </c>
       <c r="M205" s="71" t="n">
@@ -31925,7 +31231,12 @@
       </c>
       <c r="U205" t="inlineStr">
         <is>
-          <t>/composition/layers/100/clips/1/video/opacity</t>
+          <t>/composition/layers/100/clips/1/connect</t>
+        </is>
+      </c>
+      <c r="X205" t="inlineStr">
+        <is>
+          <t>Connected=1; Disconnected=1</t>
         </is>
       </c>
     </row>
@@ -31933,11 +31244,7 @@
       <c r="A206" s="71" t="n">
         <v>202</v>
       </c>
-      <c r="B206" s="72" t="inlineStr">
-        <is>
-          <t>1784313902100</t>
-        </is>
-      </c>
+      <c r="B206" s="72" t="n"/>
       <c r="C206" t="inlineStr">
         <is>
           <t>motion_y</t>
@@ -31979,7 +31286,7 @@
       </c>
       <c r="L206" t="inlineStr">
         <is>
-          <t>/composition/layers/100/clips/1/video/effects/transform/positiony</t>
+          <t>/composition/layers/100/clips/1/connect</t>
         </is>
       </c>
       <c r="M206" s="71" t="n">
@@ -32009,7 +31316,12 @@
       </c>
       <c r="U206" t="inlineStr">
         <is>
-          <t>/composition/layers/100/clips/1/video/effects/transform/positiony</t>
+          <t>/composition/layers/100/clips/1/connect</t>
+        </is>
+      </c>
+      <c r="X206" t="inlineStr">
+        <is>
+          <t>Connected=1; Disconnected=1</t>
         </is>
       </c>
     </row>
@@ -32017,11 +31329,7 @@
       <c r="A207" s="71" t="n">
         <v>203</v>
       </c>
-      <c r="B207" s="72" t="inlineStr">
-        <is>
-          <t>1784313900123</t>
-        </is>
-      </c>
+      <c r="B207" s="72" t="n"/>
       <c r="C207" t="inlineStr">
         <is>
           <t>button_connect</t>

</xml_diff>